<commit_message>
🔄 Auto-refresh: 2026-04-07 22:39 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$154</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1082,12 +1082,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>Glocomms</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1115,19 +1115,19 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Data Analyst – Business Data Analyst (with Experience)</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NewCo Capital Group</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1155,19 +1155,19 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst – Business Data Analyst (with Experience)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>NewCo Capital Group</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1195,19 +1195,19 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1235,19 +1235,19 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>LSC - LifeSciences Consultants</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1275,58 +1275,54 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>LSC - LifeSciences Consultants</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
-        </is>
-      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1341,7 +1337,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1358,19 +1354,19 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1385,7 +1381,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1402,19 +1398,19 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1446,19 +1442,19 @@
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1473,7 +1469,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1490,24 +1486,24 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1517,7 +1513,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1534,24 +1530,24 @@
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1561,7 +1557,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1578,19 +1574,19 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1605,7 +1601,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1627,19 +1623,19 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1649,7 +1645,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1666,39 +1662,39 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1708,22 +1704,26 @@
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Data Scientist (Analyst)</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Why Hiring</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1751,7 +1751,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-analyst-at-why-hiring-4397930157</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
@@ -1798,12 +1798,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Business Intelligence Reporting Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>StepStone Group</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>La Jolla, CA</t>
+          <t>Connecticut, United States</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1831,19 +1831,19 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-reporting-analyst-at-stepstone-group-4394490796</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Reporting Analyst</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>StepStone Group</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>La Jolla, CA</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1871,7 +1871,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-reporting-analyst-at-stepstone-group-4394490796</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>FNS, Inc.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Torrance, CA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -1911,19 +1911,19 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -1951,19 +1951,19 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Business Analyst III (Supply Chain Optimization): 26-00856</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>US Alliance Group, Inc</t>
+          <t>Akraya, Inc.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Rancho Santa Margarita, CA</t>
+          <t>North Reading, MA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -1991,29 +1991,29 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-us-alliance-group-inc-4397387940</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-iii-supply-chain-optimization-26-00856-at-akraya-inc-4398091020</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -2031,29 +2031,29 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2071,19 +2071,19 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>US Alliance Group, Inc</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Rancho Santa Margarita, CA</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2111,29 +2111,29 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-us-alliance-group-inc-4397387940</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2151,19 +2151,19 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2173,129 +2173,117 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2293,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2322,24 +2310,24 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2349,7 +2337,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2366,24 +2354,24 @@
       <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2393,7 +2381,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2410,24 +2398,24 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2437,7 +2425,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2454,39 +2442,39 @@
       <c r="H48" s="2" t="inlineStr"/>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2496,37 +2484,41 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>1stDibs</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2536,37 +2528,41 @@
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2576,22 +2572,26 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2619,29 +2619,29 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Business Analyst I (Full Time) United States</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>1stDibs</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2659,107 +2659,99 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
-        </is>
-      </c>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Business Analyst I (Full Time) United States</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2769,41 +2761,37 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
-        </is>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2813,7 +2801,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2830,19 +2818,19 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2857,7 +2845,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2874,19 +2862,19 @@
       <c r="H58" s="2" t="inlineStr"/>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2901,7 +2889,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2918,39 +2906,39 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2960,37 +2948,41 @@
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+        </is>
+      </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3000,22 +2992,26 @@
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3025,12 +3021,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3040,22 +3036,26 @@
       </c>
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3083,19 +3083,19 @@
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>AutoPayPlus</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3123,29 +3123,29 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3163,19 +3163,19 @@
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Marchon Partners</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3203,19 +3203,19 @@
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Robert Half</t>
+          <t>AutoPayPlus</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Orlando, FL</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3243,19 +3243,19 @@
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-robert-half-4395319491</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3265,60 +3265,52 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3326,23 +3318,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3374,19 +3370,19 @@
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3401,7 +3397,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3418,19 +3414,19 @@
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3445,7 +3441,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3462,19 +3458,19 @@
       <c r="H72" s="2" t="inlineStr"/>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3489,7 +3485,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3506,24 +3502,24 @@
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3533,7 +3529,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -3550,24 +3546,24 @@
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3577,7 +3573,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3594,19 +3590,19 @@
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Marketing</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3621,7 +3617,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3643,14 +3639,14 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5161402008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3665,7 +3661,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3687,14 +3683,14 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5161402008</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3731,14 +3727,14 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3775,19 +3771,19 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3797,7 +3793,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3814,19 +3810,19 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3841,7 +3837,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3863,19 +3859,19 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3885,7 +3881,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3902,19 +3898,19 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3929,7 +3925,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3946,19 +3942,19 @@
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3973,7 +3969,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3990,19 +3986,19 @@
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4017,7 +4013,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4039,14 +4035,14 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4061,7 +4057,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4078,19 +4074,19 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4122,19 +4118,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4149,7 +4145,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4166,19 +4162,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4193,7 +4189,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4215,14 +4211,14 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4237,7 +4233,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4254,19 +4250,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4281,7 +4277,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4298,19 +4294,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4325,7 +4321,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4342,19 +4338,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4369,7 +4365,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4386,19 +4382,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4413,7 +4409,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4430,19 +4426,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Risk &amp; Control Health Data Analyst</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4457,7 +4453,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4474,19 +4470,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4501,7 +4497,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4518,19 +4514,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4545,7 +4541,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4562,39 +4558,39 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>iHeartMedia</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -4604,22 +4600,26 @@
       </c>
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr"/>
-      <c r="I98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+        </is>
+      </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>(USA) Data Analyst II</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VIZIO</t>
+          <t>iHeartMedia</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4647,19 +4647,19 @@
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>(USA) Data Analyst II</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Shaw Industries</t>
+          <t>VIZIO</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Dalton, GA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4687,29 +4687,29 @@
       <c r="I100" s="2" t="inlineStr"/>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-shaw-industries-4396260014</t>
+          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Data Scientist, All Levels</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>Shaw Industries</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dalton, GA</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4727,29 +4727,29 @@
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-shaw-industries-4396260014</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Data Scientist, All Levels</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Orchard</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4767,19 +4767,19 @@
       <c r="I102" s="2" t="inlineStr"/>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-orchard-4396257878</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Curana Health</t>
+          <t>Orchard</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4807,19 +4807,19 @@
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-curana-health-4396245139</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-orchard-4396257878</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Curana Health</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -4829,36 +4829,32 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr"/>
-      <c r="I104" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
-        </is>
-      </c>
+      <c r="I104" s="2" t="inlineStr"/>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-curana-health-4396245139</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4873,7 +4869,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4890,19 +4886,19 @@
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592301?gh_jid=7592301</t>
+          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4934,19 +4930,19 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7592301?gh_jid=7592301</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4961,7 +4957,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4978,19 +4974,19 @@
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5005,7 +5001,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5027,19 +5023,19 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Toyota North America</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5049,12 +5045,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Plano, TX</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5064,22 +5060,26 @@
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+        </is>
+      </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-toyota-north-america-4393967481</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Shipt</t>
+          <t>Toyota North America</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Plano, TX</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5107,58 +5107,54 @@
       <c r="I110" s="2" t="inlineStr"/>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-shipt-4393976495</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-toyota-north-america-4393967481</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Shipt</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
-        </is>
-      </c>
+      <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-shipt-4393976495</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5190,19 +5186,19 @@
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5234,24 +5230,24 @@
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5261,7 +5257,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5271,31 +5267,31 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5305,7 +5301,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5315,26 +5311,26 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5349,7 +5345,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5371,19 +5367,19 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5393,7 +5389,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5403,31 +5399,31 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -5437,7 +5433,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5454,24 +5450,24 @@
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5481,7 +5477,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5491,26 +5487,26 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -5547,29 +5543,29 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5579,41 +5575,41 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5623,31 +5619,31 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5657,7 +5653,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5674,19 +5670,19 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -5701,7 +5697,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5718,24 +5714,24 @@
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5745,7 +5741,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5755,26 +5751,26 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -5789,7 +5785,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5811,14 +5807,14 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5855,19 +5851,19 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -5877,7 +5873,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5894,19 +5890,19 @@
       <c r="H128" s="2" t="inlineStr"/>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5938,19 +5934,19 @@
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5965,7 +5961,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -5982,19 +5978,19 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -6009,7 +6005,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6026,24 +6022,24 @@
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -6053,7 +6049,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6063,26 +6059,26 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6097,7 +6093,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6107,31 +6103,31 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -6141,7 +6137,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6151,26 +6147,26 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6185,7 +6181,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6195,7 +6191,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
@@ -6207,14 +6203,14 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6229,7 +6225,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6239,7 +6235,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
@@ -6251,19 +6247,19 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6273,7 +6269,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6283,26 +6279,26 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -6317,7 +6313,7 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -6334,19 +6330,19 @@
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6361,7 +6357,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6371,26 +6367,26 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6422,19 +6418,19 @@
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6466,19 +6462,19 @@
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -6493,7 +6489,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -6510,19 +6506,19 @@
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6537,7 +6533,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6554,19 +6550,19 @@
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -6581,7 +6577,7 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -6598,24 +6594,24 @@
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6625,99 +6621,99 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="G146" s="2" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H146" s="2" t="inlineStr"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6727,26 +6723,26 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -6761,7 +6757,7 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -6771,7 +6767,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr"/>
@@ -6783,14 +6779,14 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6815,7 +6811,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="G149" t="inlineStr"/>
@@ -6827,19 +6823,19 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Figma</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -6849,7 +6845,7 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
@@ -6859,26 +6855,26 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr"/>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6915,14 +6911,14 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Scientist  </t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -6947,7 +6943,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr"/>
@@ -6959,14 +6955,14 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -7003,12 +6999,56 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer, Machine Learning</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA • New York, NY • United States</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr"/>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
           <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J153"/>
+  <autoFilter ref="A1:J154"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 02:17 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J154"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -782,51 +782,47 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -863,14 +859,14 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463699002?gh_jid=8463699002</t>
+          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -907,14 +903,14 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.brex.com/careers/8463699002?gh_jid=8463699002</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -929,7 +925,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Salt Lake City, Utah, United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -951,14 +947,14 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485388002?gh_jid=8485388002</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -973,7 +969,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Salt Lake City, Utah, United States</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -995,34 +991,34 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.brex.com/careers/8485388002?gh_jid=8485388002</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Junior Data Scientist</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Illinois, United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1032,22 +1028,26 @@
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4394781668</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Junior Data Scientist</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KellyMitchell Group</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Greenwood Village, CO</t>
+          <t>Illinois, United States</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1075,7 +1075,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4392306642</t>
+          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4394781668</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Glocomms</t>
+          <t>KellyMitchell Group</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Greenwood Village, CO</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1115,19 +1115,19 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4392306642</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>Glocomms</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1155,19 +1155,19 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst – Business Data Analyst (with Experience)</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>NewCo Capital Group</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1195,19 +1195,19 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst – Business Data Analyst (with Experience)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>NewCo Capital Group</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1235,19 +1235,19 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1275,19 +1275,19 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>LSC - LifeSciences Consultants</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1315,102 +1315,94 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
-        </is>
-      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>LSC - LifeSciences Consultants</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
-        </is>
-      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1425,7 +1417,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1442,19 +1434,19 @@
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1469,7 +1461,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1486,19 +1478,19 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1513,7 +1505,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1530,24 +1522,24 @@
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1557,7 +1549,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1574,24 +1566,24 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1601,7 +1593,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1618,24 +1610,24 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1645,7 +1637,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1662,24 +1654,24 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1689,7 +1681,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1706,39 +1698,39 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1748,37 +1740,41 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1788,22 +1784,26 @@
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Connecticut, United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1831,19 +1831,19 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Reporting Analyst</t>
+          <t>Machine Learning Engineer I</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>StepStone Group</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>La Jolla, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1871,19 +1871,19 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-reporting-analyst-at-stepstone-group-4394490796</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>FNS, Inc.</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Connecticut, United States</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1911,19 +1911,19 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>RadNet</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1951,19 +1951,19 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Business Analyst III (Supply Chain Optimization): 26-00856</t>
+          <t>Business Intelligence Reporting Analyst</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Akraya, Inc.</t>
+          <t>StepStone Group</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>North Reading, MA</t>
+          <t>La Jolla, CA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1991,7 +1991,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-iii-supply-chain-optimization-26-00856-at-akraya-inc-4398091020</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-reporting-analyst-at-stepstone-group-4394490796</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>FNS, Inc.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Torrance, CA</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -2031,19 +2031,19 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -2071,19 +2071,19 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>US Alliance Group, Inc</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Rancho Santa Margarita, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
@@ -2111,29 +2111,29 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-us-alliance-group-inc-4397387940</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2151,29 +2151,29 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>AEG</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2191,29 +2191,29 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2231,29 +2231,29 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2271,107 +2271,99 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2381,7 +2373,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2398,24 +2390,24 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2425,7 +2417,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2442,24 +2434,24 @@
       <c r="H48" s="2" t="inlineStr"/>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2469,7 +2461,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2486,19 +2478,19 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2513,7 +2505,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2535,14 +2527,14 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2557,7 +2549,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2579,34 +2571,34 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2616,10 +2608,14 @@
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2627,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1stDibs</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2659,19 +2655,19 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>1stDibs</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2681,7 +2677,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2699,19 +2695,19 @@
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2721,7 +2717,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2739,7 +2735,7 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4009,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4030,12 +4026,12 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4522,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4558,19 +4554,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4585,7 +4581,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4602,39 +4598,39 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>iHeartMedia</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4644,22 +4640,26 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+        </is>
+      </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>(USA) Data Analyst II</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>VIZIO</t>
+          <t>iHeartMedia</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -4687,19 +4687,19 @@
       <c r="I100" s="2" t="inlineStr"/>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>(USA) Data Analyst II</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Shaw Industries</t>
+          <t>VIZIO</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4709,7 +4709,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Dalton, GA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4727,29 +4727,29 @@
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-shaw-industries-4396260014</t>
+          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, All Levels</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>Shaw Industries</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dalton, GA</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4767,29 +4767,29 @@
       <c r="I102" s="2" t="inlineStr"/>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-shaw-industries-4396260014</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Data Scientist, All Levels</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Orchard</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4807,19 +4807,19 @@
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-orchard-4396257878</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Curana Health</t>
+          <t>Orchard</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4847,7 +4847,7 @@
       <c r="I104" s="2" t="inlineStr"/>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-curana-health-4396245139</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-orchard-4396257878</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592301?gh_jid=7592301</t>
+          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
         </is>
       </c>
     </row>
@@ -5074,87 +5074,95 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Toyota North America</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Plano, TX</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr"/>
-      <c r="I110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+        </is>
+      </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-toyota-north-america-4393967481</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Shipt</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+        </is>
+      </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-shipt-4393976495</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5186,24 +5194,24 @@
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5213,7 +5221,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5223,31 +5231,31 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5257,7 +5265,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5267,31 +5275,31 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5301,7 +5309,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5311,31 +5319,31 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -5345,7 +5353,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5355,31 +5363,31 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5389,7 +5397,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5399,31 +5407,31 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -5433,7 +5441,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5443,31 +5451,31 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5477,7 +5485,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5487,41 +5495,41 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -5531,31 +5539,31 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr"/>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5565,7 +5573,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5575,41 +5583,41 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5619,31 +5627,31 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5653,7 +5661,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5670,24 +5678,24 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -5697,7 +5705,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5707,31 +5715,31 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5741,7 +5749,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5751,26 +5759,26 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -5785,7 +5793,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5807,19 +5815,19 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5829,7 +5837,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5846,24 +5854,24 @@
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -5873,7 +5881,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5890,19 +5898,19 @@
       <c r="H128" s="2" t="inlineStr"/>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5917,7 +5925,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5934,19 +5942,19 @@
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5978,24 +5986,24 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6005,7 +6013,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6015,31 +6023,31 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -6049,7 +6057,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6059,31 +6067,31 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -6093,7 +6101,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6103,31 +6111,31 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -6137,7 +6145,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6147,26 +6155,26 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6181,7 +6189,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6191,7 +6199,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
@@ -6203,19 +6211,19 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -6225,7 +6233,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6235,31 +6243,31 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6269,7 +6277,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6279,26 +6287,26 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -6313,7 +6321,7 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -6323,26 +6331,26 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr"/>
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6357,7 +6365,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6367,26 +6375,26 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6418,19 +6426,19 @@
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6445,7 +6453,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6462,19 +6470,19 @@
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -6506,19 +6514,19 @@
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6533,7 +6541,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6550,24 +6558,24 @@
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -6577,51 +6585,55 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="G144" s="2" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6631,31 +6643,31 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -6665,55 +6677,51 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G146" s="2" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr"/>
       <c r="H146" s="2" t="inlineStr"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6723,26 +6731,26 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -6757,7 +6765,7 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -6767,7 +6775,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr"/>
@@ -6779,19 +6787,19 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6801,7 +6809,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6811,31 +6819,31 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -6845,7 +6853,7 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
@@ -6855,26 +6863,26 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr"/>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6899,7 +6907,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="G151" t="inlineStr"/>
@@ -6911,14 +6919,14 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t>Software Engineer, Machine Learning</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -6943,7 +6951,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr"/>
@@ -6955,100 +6963,12 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data Scientist  </t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>Figma</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer, Machine Learning</t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="inlineStr">
-        <is>
-          <t>Figma</t>
-        </is>
-      </c>
-      <c r="C154" s="2" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="G154" s="2" t="inlineStr"/>
-      <c r="H154" s="2" t="inlineStr"/>
-      <c r="I154" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J154" s="2" t="inlineStr">
-        <is>
           <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J154"/>
+  <autoFilter ref="A1:J152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 07:19 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Posted 7 D</t>
+          <t>Posted 8 D</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -567,7 +567,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Posted 6 D</t>
+          <t>Posted 7 D</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posted 19 </t>
+          <t xml:space="preserve">Posted 20 </t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posted 13 </t>
+          <t xml:space="preserve">Posted 14 </t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1498,12 +1498,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>LSC - LifeSciences Consultants</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1531,19 +1531,19 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>LSC - LifeSciences Consultants</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1571,7 +1571,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>FNS, Inc.</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2123,7 +2123,7 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2163,19 +2163,19 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
@@ -2203,7 +2203,7 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>AEG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,29 +2243,29 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,19 +2283,19 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,29 +2323,29 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2363,7 +2363,7 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2403,54 +2403,58 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2465,7 +2469,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2487,19 +2491,19 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2509,7 +2513,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2526,24 +2530,24 @@
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2553,7 +2557,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2570,12 +2574,12 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
@@ -3418,12 +3422,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Marchon Partners</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3433,60 +3437,52 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3494,23 +3490,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3542,19 +3542,19 @@
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3586,19 +3586,19 @@
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3630,19 +3630,19 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3674,24 +3674,24 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3718,24 +3718,24 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3762,19 +3762,19 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3811,14 +3811,14 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3899,19 +3899,19 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3938,19 +3938,19 @@
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3987,19 +3987,19 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4026,19 +4026,19 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4070,19 +4070,19 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4114,19 +4114,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4163,14 +4163,14 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4202,19 +4202,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4246,19 +4246,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4290,19 +4290,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4339,14 +4339,14 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4378,19 +4378,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4422,19 +4422,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4466,19 +4466,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4510,19 +4510,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4554,19 +4554,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Risk &amp; Control Health Data Analyst</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4598,19 +4598,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
@@ -4862,12 +4862,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Orchard</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4895,19 +4895,19 @@
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-orchard-4396257878</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382819672</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -4917,32 +4917,36 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
-      <c r="I106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
+        </is>
+      </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382819672</t>
+          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4974,19 +4978,19 @@
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
+          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5001,7 +5005,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5018,19 +5022,19 @@
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5045,7 +5049,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5062,19 +5066,19 @@
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5089,7 +5093,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5111,29 +5115,29 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5143,26 +5147,26 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5194,19 +5198,19 @@
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5238,24 +5242,24 @@
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5265,7 +5269,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5275,31 +5279,31 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5309,7 +5313,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5319,26 +5323,26 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5353,7 +5357,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5375,19 +5379,19 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5397,7 +5401,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5407,31 +5411,31 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -5441,7 +5445,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5458,24 +5462,24 @@
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5485,7 +5489,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5495,26 +5499,26 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -5551,29 +5555,29 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5583,41 +5587,41 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5627,31 +5631,31 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735255&amp;gh_jid=7735255</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5661,7 +5665,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5678,24 +5682,24 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735255&amp;gh_jid=7735255</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -5705,7 +5709,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5715,26 +5719,26 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5749,7 +5753,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5771,14 +5775,14 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -5815,19 +5819,19 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5837,7 +5841,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5854,19 +5858,19 @@
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -5881,7 +5885,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5898,24 +5902,24 @@
       <c r="H128" s="2" t="inlineStr"/>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5925,7 +5929,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5935,26 +5939,26 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5969,7 +5973,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -5979,31 +5983,31 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6013,7 +6017,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6023,26 +6027,26 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6057,7 +6061,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6067,7 +6071,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
@@ -6079,14 +6083,14 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6101,7 +6105,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6111,7 +6115,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
@@ -6123,19 +6127,19 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -6145,7 +6149,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6155,26 +6159,26 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6189,7 +6193,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6206,19 +6210,19 @@
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6233,7 +6237,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6243,26 +6247,26 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6294,19 +6298,19 @@
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -6338,19 +6342,19 @@
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6365,7 +6369,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6382,19 +6386,19 @@
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6409,7 +6413,7 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -6426,19 +6430,19 @@
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6453,7 +6457,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6470,24 +6474,24 @@
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -6497,99 +6501,99 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="G142" s="2" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -6599,26 +6603,26 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -6633,7 +6637,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6643,7 +6647,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
@@ -6655,14 +6659,14 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -6687,7 +6691,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
@@ -6699,19 +6703,19 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6721,7 +6725,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6731,26 +6735,26 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -6787,14 +6791,14 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6819,7 +6823,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="G149" t="inlineStr"/>
@@ -6831,14 +6835,14 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Scientist  </t>
+          <t>Software Engineer, Machine Learning</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -6875,56 +6879,12 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Software Engineer, Machine Learning</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Figma</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="G151" t="inlineStr"/>
-      <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
           <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J151"/>
+  <autoFilter ref="A1:J150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 09:01 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>KellyMitchell Group</t>
+          <t>Glocomms</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Greenwood Village, CO</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1291,19 +1291,19 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4392306642</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Glocomms</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1331,19 +1331,19 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Data Analyst – Business Data Analyst (with Experience)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>NewCo Capital Group</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1371,19 +1371,19 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Data Analyst – Business Data Analyst (with Experience)</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NewCo Capital Group</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1411,19 +1411,19 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1451,19 +1451,19 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1491,19 +1491,19 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>LSC - LifeSciences Consultants</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1531,54 +1531,58 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LSC - LifeSciences Consultants</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1593,7 +1597,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1610,19 +1614,19 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1637,7 +1641,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1654,19 +1658,19 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1698,19 +1702,19 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1725,7 +1729,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1742,24 +1746,24 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1769,7 +1773,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1786,24 +1790,24 @@
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1813,7 +1817,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1830,19 +1834,19 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1857,7 +1861,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1879,34 +1883,34 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1916,26 +1920,22 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Machine Learning Engineer I</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1963,19 +1963,19 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Connecticut, United States</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2003,19 +2003,19 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>RadNet</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Connecticut, United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2043,19 +2043,19 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RadNet</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2083,7 +2083,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
@@ -2123,19 +2123,19 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2163,7 +2163,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>AEG</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2203,29 +2203,29 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,19 +2243,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,29 +2283,29 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,7 +2323,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2363,54 +2363,58 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2425,7 +2429,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2447,19 +2451,19 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2469,7 +2473,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2486,24 +2490,24 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2513,7 +2517,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2530,24 +2534,24 @@
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2557,7 +2561,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2574,19 +2578,19 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2601,7 +2605,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2623,14 +2627,14 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2645,7 +2649,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2667,34 +2671,34 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2704,14 +2708,10 @@
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>1stDibs</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2751,19 +2751,19 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>1stDibs</t>
+          <t>KellyMitchell Group</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Irving, TX</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2791,7 +2791,7 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4397306957</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735255&amp;gh_jid=7735255</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 10:56 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -958,12 +958,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>University of Iowa</t>
+          <t>SeatGeek</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Iowa City, IA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -991,63 +991,59 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1057,36 +1053,32 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463699002?gh_jid=8463699002</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1123,14 +1115,14 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1145,7 +1137,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Salt Lake City, Utah, United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1167,14 +1159,14 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485388002?gh_jid=8485388002</t>
+          <t>https://www.brex.com/careers/8463699002?gh_jid=8463699002</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1211,34 +1203,34 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Junior Data Scientist</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Illinois, United States</t>
+          <t>Salt Lake City, Utah, United States</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1248,37 +1240,41 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4394781668</t>
+          <t>https://www.brex.com/careers/8485388002?gh_jid=8485388002</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Glocomms</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1288,22 +1284,26 @@
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Junior Data Scientist</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Illinois, United States</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1331,19 +1331,19 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4394781668</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst – Business Data Analyst (with Experience)</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>NewCo Capital Group</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1371,19 +1371,19 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst – Business Data Analyst (with Experience)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>NewCo Capital Group</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1411,19 +1411,19 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1451,19 +1451,19 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1491,19 +1491,19 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>LSC - LifeSciences Consultants</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4398343669</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
@@ -1930,12 +1930,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1963,19 +1963,19 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Machine Learning Engineer I</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Connecticut, United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2003,19 +2003,19 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>RadNet</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Connecticut, United States</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2043,19 +2043,19 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>RadNet</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2083,7 +2083,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
@@ -2123,19 +2123,19 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2163,7 +2163,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2203,29 +2203,29 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>AEG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,19 +2243,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,29 +2283,29 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,7 +2323,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2363,58 +2363,54 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2429,7 +2425,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2451,19 +2447,19 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2473,7 +2469,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2490,24 +2486,24 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2517,7 +2513,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2534,24 +2530,24 @@
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2561,7 +2557,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2578,19 +2574,19 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2605,7 +2601,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2627,14 +2623,14 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2649,7 +2645,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2671,34 +2667,34 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2708,10 +2704,14 @@
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1stDibs</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2751,19 +2751,19 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>KellyMitchell Group</t>
+          <t>1stDibs</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Irving, TX</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2791,19 +2791,19 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4397306957</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>KellyMitchell Group</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Irving, TX</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2831,19 +2831,19 @@
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4397306957</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2871,29 +2871,29 @@
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Business Analyst I (Full Time) United States</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2911,19 +2911,19 @@
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>Business Analyst I (Full Time) United States</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2933,41 +2933,37 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2977,7 +2973,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2994,19 +2990,19 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3021,7 +3017,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3038,19 +3034,19 @@
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3065,7 +3061,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3082,19 +3078,19 @@
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3109,7 +3105,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3126,19 +3122,19 @@
       <c r="H64" s="2" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3153,7 +3149,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3170,39 +3166,39 @@
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3212,22 +3208,26 @@
       </c>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3255,29 +3255,29 @@
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3295,29 +3295,29 @@
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3335,7 +3335,7 @@
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>AutoPayPlus</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3375,19 +3375,19 @@
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>AutoPayPlus</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>Orlando, FL</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3415,19 +3415,19 @@
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Marchon Partners</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3455,19 +3455,19 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Marchon Partners</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3477,104 +3477,92 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Robert Half</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
-        </is>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-robert-half-4395319491</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3582,23 +3570,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3613,7 +3605,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3630,19 +3622,19 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3657,7 +3649,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3674,19 +3666,19 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3701,7 +3693,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3718,24 +3710,24 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3745,7 +3737,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3762,24 +3754,24 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3789,7 +3781,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3806,24 +3798,24 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3833,7 +3825,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3850,19 +3842,19 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3877,7 +3869,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3899,14 +3891,14 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3943,19 +3935,19 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3965,7 +3957,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3982,24 +3974,24 @@
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4009,7 +4001,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4026,24 +4018,24 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4053,7 +4045,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4070,24 +4062,24 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4097,7 +4089,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4114,19 +4106,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4141,7 +4133,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4158,19 +4150,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4185,7 +4177,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4202,19 +4194,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4229,7 +4221,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4246,19 +4238,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4273,7 +4265,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4295,14 +4287,14 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4317,7 +4309,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4334,19 +4326,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4361,7 +4353,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4378,19 +4370,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4422,19 +4414,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4449,7 +4441,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4466,19 +4458,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4493,7 +4485,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4510,19 +4502,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4537,7 +4529,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4554,19 +4546,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4581,7 +4573,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4598,19 +4590,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4625,7 +4617,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4642,19 +4634,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Risk &amp; Control Health Data Analyst</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4669,7 +4661,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4686,19 +4678,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4713,7 +4705,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4730,39 +4722,39 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>iHeartMedia</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -4772,37 +4764,41 @@
       </c>
       <c r="G102" s="2" t="inlineStr"/>
       <c r="H102" s="2" t="inlineStr"/>
-      <c r="I102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+        </is>
+      </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>(USA) Data Analyst II</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VIZIO</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4812,32 +4808,36 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+        </is>
+      </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, All Levels</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>iHeartMedia</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4855,19 +4855,19 @@
       <c r="I104" s="2" t="inlineStr"/>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>(USA) Data Analyst II</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>VIZIO</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4895,58 +4895,54 @@
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382819672</t>
+          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Data Scientist, All Levels</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
-        </is>
-      </c>
+      <c r="I106" s="2" t="inlineStr"/>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4978,19 +4974,19 @@
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
+          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5005,7 +5001,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5022,19 +5018,19 @@
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5049,7 +5045,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5066,19 +5062,19 @@
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5093,7 +5089,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5115,29 +5111,29 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5147,26 +5143,26 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5198,19 +5194,19 @@
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5242,24 +5238,24 @@
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5269,7 +5265,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5279,31 +5275,31 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5313,7 +5309,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5323,26 +5319,26 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5357,7 +5353,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5379,19 +5375,19 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5401,7 +5397,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5411,31 +5407,31 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -5445,7 +5441,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5462,24 +5458,24 @@
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5489,7 +5485,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5499,26 +5495,26 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -5555,29 +5551,29 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5587,41 +5583,41 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5631,31 +5627,31 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5665,7 +5661,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5682,24 +5678,24 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -5709,7 +5705,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5719,26 +5715,26 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5753,7 +5749,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5775,14 +5771,14 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -5819,19 +5815,19 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5841,7 +5837,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5858,19 +5854,19 @@
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -5885,7 +5881,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5902,24 +5898,24 @@
       <c r="H128" s="2" t="inlineStr"/>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5929,7 +5925,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5939,26 +5935,26 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5973,7 +5969,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -5983,31 +5979,31 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6017,7 +6013,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6027,26 +6023,26 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6061,7 +6057,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6071,7 +6067,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
@@ -6083,14 +6079,14 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6105,7 +6101,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6115,7 +6111,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
@@ -6127,19 +6123,19 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -6149,7 +6145,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6159,26 +6155,26 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6193,7 +6189,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6210,19 +6206,19 @@
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6237,7 +6233,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6247,26 +6243,26 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6298,19 +6294,19 @@
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -6342,19 +6338,19 @@
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6369,7 +6365,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6386,19 +6382,19 @@
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6413,7 +6409,7 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -6430,19 +6426,19 @@
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6457,7 +6453,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6474,24 +6470,24 @@
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -6501,99 +6497,99 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G142" s="2" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -6603,26 +6599,26 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -6637,7 +6633,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6647,7 +6643,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
@@ -6659,14 +6655,14 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -6691,7 +6687,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
@@ -6703,19 +6699,19 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Figma</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6725,7 +6721,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6735,26 +6731,26 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -6791,14 +6787,14 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Scientist  </t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6823,7 +6819,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G149" t="inlineStr"/>
@@ -6835,14 +6831,14 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -6879,12 +6875,56 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Software Engineer, Machine Learning</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>San Francisco, CA • New York, NY • United States</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
           <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J150"/>
+  <autoFilter ref="A1:J151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 15:11 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -998,12 +998,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Junior Data Scientist</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Betterment</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Texas, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1031,19 +1031,19 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Junior Data Scientist</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>Texas, United States</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1071,19 +1071,19 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>University of Iowa</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Iowa City, IA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1111,29 +1111,29 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384776881</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Business Analyst - Private Capital</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Brain Co.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco Bay Area</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1151,107 +1151,99 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463699002?gh_jid=8463699002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1261,36 +1253,32 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1305,7 +1293,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Salt Lake City, Utah, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1327,14 +1315,14 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485388002?gh_jid=8485388002</t>
+          <t>https://www.brex.com/careers/8463702002?gh_jid=8463702002</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1349,7 +1337,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1371,34 +1359,34 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KellyMitchell Group</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Greenwood Village, CO</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1408,37 +1396,41 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4392306642</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Glocomms</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Seattle, Washington, United States</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1448,37 +1440,41 @@
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-glocomms-4398419364</t>
+          <t>https://www.brex.com/careers/8485386002?gh_jid=8485386002</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1488,22 +1484,26 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst – Business Data Analyst (with Experience)</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>NewCo Capital Group</t>
+          <t>KellyMitchell Group</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Greenwood Village, CO</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1531,19 +1531,19 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-%E2%80%93-business-data-analyst-with-experience-at-newco-capital-group-4398587477</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4392306642</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1571,19 +1571,19 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1611,19 +1611,19 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1651,58 +1651,54 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
-        </is>
-      </c>
+      <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1717,7 +1713,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1734,19 +1730,19 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1761,7 +1757,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1778,19 +1774,19 @@
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1822,19 +1818,19 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1849,7 +1845,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1866,24 +1862,24 @@
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1893,7 +1889,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1910,24 +1906,24 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1937,7 +1933,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1954,19 +1950,19 @@
       <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1981,7 +1977,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2003,34 +1999,34 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2040,22 +2036,26 @@
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2083,19 +2083,19 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2123,19 +2123,19 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Machine Learning Engineer I</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Connecticut, United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2163,19 +2163,19 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>RadNet</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Connecticut, United States</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2203,19 +2203,19 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Business Intelligence Reporting Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>StepStone Group</t>
+          <t>RadNet</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>La Jolla, CA</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,7 +2243,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-reporting-analyst-at-stepstone-group-4394490796</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>FNS, Inc.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>Torrance, CA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,7 +2283,7 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2323,19 +2323,19 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
@@ -2363,7 +2363,7 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2403,29 +2403,29 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>AEG</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2443,19 +2443,19 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2483,29 +2483,29 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2523,7 +2523,7 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2563,58 +2563,54 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2629,7 +2625,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2651,19 +2647,19 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2673,7 +2669,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2690,24 +2686,24 @@
       <c r="H54" s="2" t="inlineStr"/>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2717,7 +2713,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2734,24 +2730,24 @@
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2761,7 +2757,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2778,19 +2774,19 @@
       <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2805,7 +2801,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2827,14 +2823,14 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2849,7 +2845,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2871,34 +2867,34 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2908,10 +2904,14 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>1stDibs</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2951,19 +2951,19 @@
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>1stDibs</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2991,29 +2991,29 @@
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst I (Full Time) United States</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3031,63 +3031,59 @@
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>Business Analyst I (Full Time) United States</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3097,41 +3093,37 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
-        </is>
-      </c>
+      <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3141,7 +3133,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3158,19 +3150,19 @@
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3185,7 +3177,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3202,19 +3194,19 @@
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3229,7 +3221,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3246,19 +3238,19 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3273,7 +3265,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3290,39 +3282,39 @@
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3332,37 +3324,41 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+        </is>
+      </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3372,32 +3368,36 @@
       </c>
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3415,19 +3415,19 @@
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3455,29 +3455,29 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>AutoPayPlus</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3495,19 +3495,19 @@
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -3535,19 +3535,19 @@
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Marchon Partners</t>
+          <t>AutoPayPlus</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Orlando, FL</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3575,19 +3575,19 @@
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3597,60 +3597,52 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr"/>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3658,23 +3650,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3706,19 +3702,19 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3733,7 +3729,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3750,19 +3746,19 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3777,7 +3773,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3794,19 +3790,19 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3821,7 +3817,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3838,24 +3834,24 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3865,7 +3861,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3882,24 +3878,24 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3909,7 +3905,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3926,19 +3922,19 @@
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3953,7 +3949,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3975,14 +3971,14 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4019,14 +4015,14 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4063,19 +4059,19 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4085,7 +4081,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4102,19 +4098,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4129,7 +4125,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4151,19 +4147,19 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4173,7 +4169,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4190,19 +4186,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4217,7 +4213,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4234,19 +4230,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4261,7 +4257,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4278,19 +4274,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4305,7 +4301,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4322,19 +4318,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4349,7 +4345,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4366,19 +4362,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4410,19 +4406,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4437,7 +4433,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4454,19 +4450,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4481,7 +4477,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4503,14 +4499,14 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4525,7 +4521,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4542,19 +4538,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4569,7 +4565,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4586,19 +4582,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4613,7 +4609,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4630,19 +4626,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4657,7 +4653,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4674,19 +4670,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4701,7 +4697,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4718,19 +4714,19 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Risk &amp; Control Health Data Analyst</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4745,7 +4741,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4762,19 +4758,19 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4789,7 +4785,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4806,19 +4802,19 @@
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -4833,7 +4829,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4850,39 +4846,39 @@
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>iHeartMedia</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4892,22 +4888,26 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>(USA) Data Analyst II</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>VIZIO</t>
+          <t>iHeartMedia</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -4935,29 +4935,29 @@
       <c r="I106" s="2" t="inlineStr"/>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Data Scientist, All Levels</t>
+          <t>(USA) Data Analyst II</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>VIZIO</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4975,7 +4975,7 @@
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4366267633</t>
+          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 17:03 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -782,12 +782,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -814,24 +814,24 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -858,24 +858,24 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -902,24 +902,24 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -946,39 +946,39 @@
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SeatGeek</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -988,37 +988,41 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Betterment</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1028,37 +1032,41 @@
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Junior Data Scientist</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Texas, United States</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1068,37 +1076,41 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Oscar Health</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1108,37 +1120,41 @@
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384776881</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1148,22 +1164,26 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Analyst - Junior</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>University of Iowa</t>
+          <t>Global Technical Talent, an Inc. 5000 Company</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1173,7 +1193,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Iowa City, IA</t>
+          <t>Framingham, MA</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1191,19 +1211,19 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>SeatGeek</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1213,7 +1233,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1231,24 +1251,24 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst - Private Capital</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Betterment</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1271,239 +1291,219 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Junior Data Scientist</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Texas, United States</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463702002?gh_jid=8463702002</t>
+          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384776881</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>North Carolina, United States</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4398606356</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Brain Co.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Seattle, Washington, United States</t>
+          <t>San Francisco Bay Area</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485386002?gh_jid=8485386002</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>C.Mendes-Engenharia, Lda</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
-        </is>
-      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-c-mendes-engenharia-lda-4399294978</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Business Intelligence Analyst (Power BI)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>KellyMitchell Group</t>
+          <t>Chadwell Supply</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Greenwood Village, CO</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1531,19 +1531,19 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4392306642</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1571,19 +1571,19 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -1611,29 +1611,29 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1651,34 +1651,34 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1688,22 +1688,26 @@
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.brex.com/careers/8463702002?gh_jid=8463702002</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1713,7 +1717,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1723,31 +1727,31 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1757,7 +1761,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1767,31 +1771,31 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1801,7 +1805,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Seattle, Washington, United States</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1811,31 +1815,31 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.brex.com/careers/8485386002?gh_jid=8485386002</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1845,7 +1849,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1855,207 +1859,191 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the AI-powered spend platform. We help companies spend with confidence with integrated corporate cards, banking, and global payments, plus intuitive software for travel and expenses. Tens of thousands of companies from startups to enterprises — including DoorDash, Flexport, and C</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Profound</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Buffalo-Niagara Falls Area</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-profound-4396666280</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2065,7 +2053,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2075,7 +2063,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -2083,34 +2071,34 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2120,37 +2108,41 @@
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2160,37 +2152,41 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Connecticut, United States</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2200,22 +2196,26 @@
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4397971257</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RadNet</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,19 +2243,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-radnet-4394711124</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>FNS, Inc.</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,19 +2283,19 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Machine Learning Engineer I</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>City of Maricopa</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Maricopa, AZ</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,7 +2323,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>City of Maricopa</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Maricopa, AZ</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
@@ -2363,19 +2363,19 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-city-of-maricopa-4397966224</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2443,7 +2443,7 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
@@ -2998,12 +2998,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>KellyMitchell Group</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Irving, TX</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3031,19 +3031,19 @@
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4397306957</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3071,7 +3071,7 @@
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
@@ -3622,12 +3622,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Marchon Partners</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3637,60 +3637,52 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3698,23 +3690,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3746,19 +3742,19 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3773,7 +3769,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3790,19 +3786,19 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3817,7 +3813,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3834,19 +3830,19 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3861,7 +3857,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3878,24 +3874,24 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3905,7 +3901,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3922,24 +3918,24 @@
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3949,7 +3945,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3966,19 +3962,19 @@
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3993,7 +3989,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4015,14 +4011,14 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4059,14 +4055,14 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4103,19 +4099,19 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4125,7 +4121,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4142,19 +4138,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4169,7 +4165,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4191,19 +4187,19 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -4213,7 +4209,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4230,19 +4226,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4257,7 +4253,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4274,19 +4270,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4301,7 +4297,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4318,19 +4314,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4345,7 +4341,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4362,19 +4358,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4389,7 +4385,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4406,19 +4402,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4450,19 +4446,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4477,7 +4473,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4494,19 +4490,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4521,7 +4517,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4543,14 +4539,14 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4565,7 +4561,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4582,19 +4578,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4609,7 +4605,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4626,19 +4622,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4653,7 +4649,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4670,19 +4666,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4697,7 +4693,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4714,19 +4710,19 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4741,7 +4737,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4758,19 +4754,19 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Risk &amp; Control Health Data Analyst</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4785,7 +4781,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4802,19 +4798,19 @@
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -4829,7 +4825,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4846,19 +4842,19 @@
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4873,7 +4869,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4890,39 +4886,39 @@
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>iHeartMedia</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -4932,22 +4928,26 @@
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
-      <c r="I106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+        </is>
+      </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>(USA) Data Analyst II</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>VIZIO</t>
+          <t>iHeartMedia</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4975,19 +4975,19 @@
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>(USA) Data Analyst II</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>VIZIO</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -4997,36 +4997,32 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
-      <c r="I108" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
-        </is>
-      </c>
+      <c r="I108" s="2" t="inlineStr"/>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
+          <t>https://www.linkedin.com/jobs/view/usa-data-analyst-ii-at-vizio-4379317924</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5058,19 +5054,19 @@
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
+          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5085,7 +5081,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5102,19 +5098,19 @@
       <c r="H110" s="2" t="inlineStr"/>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5129,7 +5125,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5146,19 +5142,19 @@
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5173,7 +5169,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -5195,29 +5191,29 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5227,26 +5223,26 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -5278,19 +5274,19 @@
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5322,24 +5318,24 @@
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -5349,7 +5345,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5359,31 +5355,31 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5393,7 +5389,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5403,26 +5399,26 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -5437,7 +5433,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5459,19 +5455,19 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5481,7 +5477,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5491,31 +5487,31 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -5525,7 +5521,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -5542,24 +5538,24 @@
       <c r="H120" s="2" t="inlineStr"/>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5569,7 +5565,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5579,26 +5575,26 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -5635,29 +5631,29 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5667,41 +5663,41 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5711,31 +5707,31 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5745,7 +5741,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5762,24 +5758,24 @@
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -5789,7 +5785,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5799,26 +5795,26 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr"/>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5833,7 +5829,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5855,14 +5851,14 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -5899,19 +5895,19 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5921,7 +5917,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5938,19 +5934,19 @@
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5965,7 +5961,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -5982,24 +5978,24 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6009,7 +6005,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6019,26 +6015,26 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6053,7 +6049,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6063,31 +6059,31 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -6097,7 +6093,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6107,26 +6103,26 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -6141,7 +6137,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6151,7 +6147,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
@@ -6163,14 +6159,14 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6185,7 +6181,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6195,7 +6191,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
@@ -6207,19 +6203,19 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -6229,7 +6225,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6239,26 +6235,26 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6273,7 +6269,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6290,19 +6286,19 @@
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -6317,7 +6313,7 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -6327,26 +6323,26 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr"/>
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6378,19 +6374,19 @@
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6422,19 +6418,19 @@
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6449,7 +6445,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6466,19 +6462,19 @@
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -6493,7 +6489,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -6510,19 +6506,19 @@
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6537,7 +6533,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6554,24 +6550,24 @@
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -6581,99 +6577,99 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G144" s="2" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
@@ -6683,26 +6679,26 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
       <c r="H146" s="2" t="inlineStr"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -6717,7 +6713,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6727,7 +6723,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
@@ -6739,14 +6735,14 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -6771,7 +6767,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr"/>
@@ -6783,19 +6779,19 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Figma</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6805,7 +6801,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6815,26 +6811,26 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -6871,14 +6867,14 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Scientist  </t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6903,7 +6899,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G151" t="inlineStr"/>
@@ -6915,14 +6911,14 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -6959,12 +6955,56 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Software Engineer, Machine Learning</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>San Francisco, CA • New York, NY • United States</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
           <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J152"/>
+  <autoFilter ref="A1:J153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-08 19:18 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -1338,12 +1338,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Junior Data Scientist</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Oscar Health</t>
+          <t>Brooksource</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Columbus, Ohio Metropolitan Area</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1371,19 +1371,19 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384776881</t>
+          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-brooksource-4396340338</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>North Carolina, United States</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1411,19 +1411,19 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4398606356</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384776881</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>North Carolina, United States</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1451,19 +1451,19 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-tech-consulting-4398606356</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C.Mendes-Engenharia, Lda</t>
+          <t>Brain Co.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco Bay Area</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1491,7 +1491,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-c-mendes-engenharia-lda-4399294978</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
+          <t>https://www.brex.com/careers/8463699002?gh_jid=8463699002</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Seattle, Washington, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485386002?gh_jid=8485386002</t>
+          <t>https://www.brex.com/careers/8485352002?gh_jid=8485352002</t>
         </is>
       </c>
     </row>
@@ -1878,12 +1878,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Profound</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Buffalo-Niagara Falls Area</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1911,19 +1911,19 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-profound-4396666280</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1951,19 +1951,19 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1991,19 +1991,19 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398554937</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2031,59 +2031,63 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2093,7 +2097,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2110,19 +2114,19 @@
       <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2137,7 +2141,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2159,34 +2163,34 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2196,26 +2200,22 @@
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,19 +2243,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Machine Learning Engineer I</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,19 +2283,19 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>FNS, Inc.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Torrance, CA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,7 +2323,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
         </is>
       </c>
     </row>
@@ -2450,22 +2450,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>AEG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2483,19 +2483,19 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-aeg-4384637228</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Agentic AI</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Zillow</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2523,29 +2523,29 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Machine Learning Engineer, Agentic AI</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2563,7 +2563,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-agentic-ai-at-zillow-4385528913</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Meltwater</t>
+          <t>Ibotta</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2603,58 +2603,54 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-ibotta-4384285582</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meltwater</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-at-meltwater-4394236575</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2669,7 +2665,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2691,19 +2687,19 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2713,7 +2709,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2730,24 +2726,24 @@
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2757,7 +2753,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2774,24 +2770,24 @@
       <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2801,7 +2797,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2818,19 +2814,19 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2845,7 +2841,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2867,14 +2863,14 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2889,7 +2885,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2911,34 +2907,34 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2948,10 +2944,14 @@
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1stDibs</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2991,19 +2991,19 @@
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>KellyMitchell Group</t>
+          <t>1stDibs</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Irving, TX</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3031,19 +3031,19 @@
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4397306957</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-1stdibs-4385170492</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>KellyMitchell Group</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Irving, TX</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3071,29 +3071,29 @@
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-at-kellymitchell-group-4397306957</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst I (Full Time) United States</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3111,63 +3111,59 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>Business Analyst I (Full Time) United States</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3177,41 +3173,37 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
-        </is>
-      </c>
+      <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-i-full-time-united-states-at-cisco-4397311380</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3221,7 +3213,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3238,19 +3230,19 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3265,7 +3257,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3282,19 +3274,19 @@
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3309,7 +3301,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3326,19 +3318,19 @@
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3353,7 +3345,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3370,39 +3362,39 @@
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3412,37 +3404,41 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+        </is>
+      </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3452,32 +3448,36 @@
       </c>
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3495,19 +3495,19 @@
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -3535,29 +3535,29 @@
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>AutoPayPlus</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3575,19 +3575,19 @@
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3615,19 +3615,19 @@
       <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Marchon Partners</t>
+          <t>AutoPayPlus</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Orlando, FL</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3655,19 +3655,19 @@
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3677,60 +3677,52 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr"/>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3738,23 +3730,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3786,19 +3782,19 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3813,7 +3809,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3830,19 +3826,19 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3857,7 +3853,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3874,19 +3870,19 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3901,7 +3897,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3918,24 +3914,24 @@
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3945,7 +3941,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3962,24 +3958,24 @@
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3989,7 +3985,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4006,19 +4002,19 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4033,7 +4029,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4055,14 +4051,14 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4099,14 +4095,14 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4143,19 +4139,19 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4165,7 +4161,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4182,19 +4178,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4209,7 +4205,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4231,19 +4227,19 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4253,7 +4249,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4270,19 +4266,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4297,7 +4293,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4314,19 +4310,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4341,7 +4337,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4358,19 +4354,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4385,7 +4381,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4402,19 +4398,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4429,7 +4425,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4446,19 +4442,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4490,19 +4486,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4517,7 +4513,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4534,19 +4530,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4561,7 +4557,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4583,14 +4579,14 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4605,7 +4601,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4622,19 +4618,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4649,7 +4645,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4666,19 +4662,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4693,7 +4689,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4710,19 +4706,19 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4737,7 +4733,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4754,19 +4750,19 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4781,7 +4777,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4798,19 +4794,19 @@
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Risk &amp; Control Health Data Analyst</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -4825,7 +4821,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4842,19 +4838,19 @@
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4869,7 +4865,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4886,19 +4882,19 @@
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4913,7 +4909,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -4930,39 +4926,39 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>iHeartMedia</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4972,10 +4968,14 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+        </is>
+      </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-iheartmedia-4383838520</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594388?gh_jid=7594388</t>
+          <t>http://www.hioscar.com/careers/7592274?gh_jid=7592274</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>Tempe, Arizona, United States</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594414?gh_jid=7594414</t>
+          <t>http://www.hioscar.com/careers/7594416?gh_jid=7594416</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Tempe, Arizona, United States</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7374162?gh_jid=7374162</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>Tempe, Arizona, United States</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7592202?gh_jid=7592202</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 02:09 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J149"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1638,12 +1638,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst (Power BI)</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chadwell Supply</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1671,19 +1671,19 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4396367708</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Business Intelligence Analyst (Power BI)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>University of Iowa</t>
+          <t>Chadwell Supply</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Iowa City, IA</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1711,19 +1711,19 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1751,29 +1751,29 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst - Private Capital</t>
+          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1791,117 +1791,109 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>Business Intelligence Analyst I</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>RemoteHunter</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-at-remotehunter-4395975249</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>MES Life Safety</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Sandy Hook, CT</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-mes-life-safety-4399227285</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>IMA Financial Group, Inc.</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1911,7 +1903,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -1919,34 +1911,34 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Entry Level Data Analyst</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1956,37 +1948,41 @@
       </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
+          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Webologix Ltd/ INC</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1996,10 +1992,14 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>HirePower Staffing Solution</t>
+          <t>IMA Financial Group, Inc.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Fullerton, CA</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2039,14 +2039,14 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Entry Level Machine Learning Engineer</t>
+          <t>Entry Level Data Analyst</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2079,19 +2079,19 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>Webologix Ltd/ INC</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2119,19 +2119,19 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CCAR Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mitchell Martin Inc.</t>
+          <t>HirePower Staffing Solution</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Jersey City, NJ</t>
+          <t>Fullerton, CA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2159,19 +2159,19 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Entry Level Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Greater Chicago Area</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2199,19 +2199,19 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Aditi Consulting</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Chillicothe, IL</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2239,19 +2239,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>CCAR Business Analyst</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>Mitchell Martin Inc.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Jersey City, NJ</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2279,19 +2279,19 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Business Analyst, Digital Media</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Taboola</t>
+          <t>Aditi Consulting</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chillicothe, IL</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2319,166 +2319,154 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-digital-media-at-taboola-4398368627</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
-        </is>
-      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Greater Chicago Area</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2488,37 +2476,41 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2528,37 +2520,41 @@
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer I</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2568,22 +2564,26 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/machine-learning-engineer-i-at-handshake-4398057615</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
@@ -2611,29 +2611,29 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -2651,107 +2651,99 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2761,41 +2753,37 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Manager, Data Science, GTM</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2805,7 +2793,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2822,24 +2810,24 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2849,7 +2837,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2866,24 +2854,24 @@
       <c r="H58" s="2" t="inlineStr"/>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2893,7 +2881,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2910,39 +2898,39 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2952,37 +2940,41 @@
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2992,22 +2984,26 @@
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3017,7 +3013,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3027,119 +3023,111 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
-        </is>
-      </c>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
-        </is>
-      </c>
+      <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3149,7 +3137,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3166,19 +3154,19 @@
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3193,7 +3181,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3210,19 +3198,19 @@
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3237,7 +3225,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3254,39 +3242,39 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3296,37 +3284,41 @@
       </c>
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+        </is>
+      </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3336,22 +3328,26 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+        </is>
+      </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3361,12 +3357,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3376,22 +3372,26 @@
       </c>
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3419,19 +3419,19 @@
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4393065831</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>AutoPayPlus</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3459,29 +3459,29 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-autopayplus-4396034123</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - SQL (SSMS)/Adv Excel</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3499,19 +3499,19 @@
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-sql-ssms-adv-excel-at-unum-4395211911</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Marchon Partners</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3521,52 +3521,60 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr"/>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-marchon-partners-4396702453</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3574,27 +3582,23 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3626,19 +3630,19 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3653,7 +3657,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3670,19 +3674,19 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3697,7 +3701,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3714,19 +3718,19 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3741,7 +3745,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3758,24 +3762,24 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3785,7 +3789,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3802,24 +3806,24 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3829,7 +3833,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3846,19 +3850,19 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3873,7 +3877,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3895,14 +3899,14 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3939,14 +3943,14 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3983,19 +3987,19 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4005,7 +4009,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4022,19 +4026,19 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4049,7 +4053,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4071,19 +4075,19 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4093,7 +4097,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4110,19 +4114,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4137,7 +4141,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4154,19 +4158,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4181,7 +4185,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4198,19 +4202,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4225,7 +4229,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4242,19 +4246,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4269,7 +4273,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4286,19 +4290,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4330,19 +4334,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4357,7 +4361,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4374,19 +4378,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4401,7 +4405,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4423,14 +4427,14 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4445,7 +4449,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4462,19 +4466,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4489,7 +4493,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4506,19 +4510,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4533,7 +4537,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4550,19 +4554,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4577,7 +4581,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4594,19 +4598,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4621,7 +4625,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4638,19 +4642,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Control Health Data Analyst</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4665,7 +4669,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4682,19 +4686,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7577621</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4709,7 +4713,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4726,19 +4730,19 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4753,7 +4757,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4770,34 +4774,34 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tempe, Arizona, United States</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4807,41 +4811,41 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>http://www.hioscar.com/careers/7594392?gh_jid=7594392</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>Tempe, Arizona, United States</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4851,31 +4855,31 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>http://www.hioscar.com/careers/7594416?gh_jid=7594416</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Data Analyst, Digital Shelf</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Kohler Co.</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4885,32 +4889,36 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Kohler, WI</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-digital-shelf-at-kohler-co-4394988521</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4925,7 +4933,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Tempe, Arizona, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -4942,19 +4950,19 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594392?gh_jid=7594392</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4969,7 +4977,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Tempe, Arizona, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4986,34 +4994,34 @@
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594416?gh_jid=7594416</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5023,41 +5031,41 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5067,41 +5075,41 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5111,31 +5119,31 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr"/>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5145,7 +5153,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5155,31 +5163,31 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -5189,7 +5197,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -5199,31 +5207,31 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5233,7 +5241,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5243,31 +5251,31 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5277,7 +5285,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5287,26 +5295,26 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5321,7 +5329,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5331,7 +5339,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
@@ -5343,14 +5351,14 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5365,7 +5373,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5375,7 +5383,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
@@ -5387,29 +5395,29 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5419,31 +5427,31 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -5453,7 +5461,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5463,31 +5471,31 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5497,7 +5505,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5507,41 +5515,41 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -5551,31 +5559,31 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr"/>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5585,7 +5593,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5595,31 +5603,31 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -5629,7 +5637,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5639,31 +5647,31 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5673,7 +5681,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5690,24 +5698,24 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -5717,7 +5725,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5734,24 +5742,24 @@
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5761,7 +5769,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5771,31 +5779,31 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -5805,7 +5813,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5815,31 +5823,31 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr"/>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5849,7 +5857,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5859,31 +5867,31 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -5893,7 +5901,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5903,31 +5911,31 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr"/>
       <c r="H128" s="2" t="inlineStr"/>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5937,7 +5945,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5947,31 +5955,31 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -5981,7 +5989,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -5991,31 +5999,31 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6025,7 +6033,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6035,31 +6043,31 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -6069,7 +6077,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6079,26 +6087,26 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6123,26 +6131,26 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -6157,7 +6165,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6167,26 +6175,26 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6201,7 +6209,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6218,19 +6226,19 @@
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6262,19 +6270,19 @@
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6289,7 +6297,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6306,24 +6314,24 @@
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
@@ -6333,51 +6341,55 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="G138" s="2" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6387,31 +6399,31 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -6421,7 +6433,7 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -6431,31 +6443,31 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr"/>
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -6465,55 +6477,51 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -6523,31 +6531,31 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6557,7 +6565,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6567,31 +6575,31 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -6601,7 +6609,7 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -6611,31 +6619,31 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6645,7 +6653,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6655,26 +6663,26 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t>Software Engineer, Machine Learning</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -6699,7 +6707,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
@@ -6711,144 +6719,48 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t>Business Analyst (Loyalty/Retention)</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Figma</t>
+          <t>Mercuryo</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>2025-12-17</t>
-        </is>
-      </c>
+          <t>Himalayas</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data Scientist  </t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
-        <is>
-          <t>Figma</t>
-        </is>
-      </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="G148" s="2" t="inlineStr"/>
-      <c r="H148" s="2" t="inlineStr"/>
-      <c r="I148" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J148" s="2" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Software Engineer, Machine Learning</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Figma</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
-        </is>
-      </c>
+          <t>Hi! We're Mercuryo , and we're on a mission to redefine finance by blending the best of traditional banking with the power of decentralized finance (DeFi). We believe everyone deserves seamless access to Web3 and traditional financial services, so we're building the platform that makes it real: one that simplifies crypto and integrates it into the broader financial ecosystem. Since launching in 20</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J149"/>
+  <autoFilter ref="A1:J147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 05:51 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2910,12 +2910,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2942,19 +2942,19 @@
       <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2991,14 +2991,14 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3035,34 +3035,34 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3072,22 +3072,26 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3097,7 +3101,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3115,63 +3119,59 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3198,19 +3198,19 @@
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3242,19 +3242,19 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3286,19 +3286,19 @@
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3330,19 +3330,19 @@
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3374,39 +3374,39 @@
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3416,22 +3416,26 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3441,7 +3445,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3459,29 +3463,29 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3499,82 +3503,74 @@
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3582,23 +3578,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3630,19 +3630,19 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3674,19 +3674,19 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3718,19 +3718,19 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3762,24 +3762,24 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3806,24 +3806,24 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3850,19 +3850,19 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3899,14 +3899,14 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3943,14 +3943,14 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3987,19 +3987,19 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4026,19 +4026,19 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4075,19 +4075,19 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4114,19 +4114,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4158,19 +4158,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4202,19 +4202,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4246,19 +4246,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4290,19 +4290,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4334,19 +4334,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4378,19 +4378,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4427,14 +4427,14 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4466,19 +4466,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4510,19 +4510,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4554,19 +4554,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4598,19 +4598,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4642,19 +4642,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735255&amp;gh_jid=7735255</t>
         </is>
       </c>
     </row>
@@ -5989,7 +5989,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6006,12 +6006,12 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>
@@ -6723,44 +6723,8 @@
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>Business Analyst (Loyalty/Retention)</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Mercuryo</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>❓ Unknown</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Himalayas</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>Hi! We're Mercuryo , and we're on a mission to redefine finance by blending the best of traditional banking with the power of decentralized finance (DeFi). We believe everyone deserves seamless access to Web3 and traditional financial services, so we're building the platform that makes it real: one that simplifies crypto and integrates it into the broader financial ecosystem. Since launching in 20</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J147"/>
+  <autoFilter ref="A1:J146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 07:22 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Posted 8 D</t>
+          <t>Posted 9 D</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -567,7 +567,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Posted 7 D</t>
+          <t>Posted 8 D</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posted 20 </t>
+          <t xml:space="preserve">Posted 21 </t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posted 14 </t>
+          <t xml:space="preserve">Posted 15 </t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -2406,12 +2406,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst, Digital Media</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>Taboola</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2439,7 +2439,7 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-digital-media-at-taboola-4398368627</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>FNS, Inc.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Torrance, CA</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
@@ -2691,19 +2691,19 @@
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -2731,29 +2731,29 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2771,19 +2771,19 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Manager, Data Science, GTM</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2793,29 +2793,25 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>New York City, NY; New York City, NY | Seattle, WA; Remote-Friendly (Travel Required) | San Francisco, CA; San Francisco, CA | New York City, NY</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5149911008</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
@@ -2910,12 +2906,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2925,7 +2921,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2942,19 +2938,19 @@
       <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2969,7 +2965,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2991,14 +2987,14 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3013,7 +3009,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3035,34 +3031,34 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3072,26 +3068,22 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3101,7 +3093,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3119,59 +3111,63 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+        </is>
+      </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3181,7 +3177,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3198,19 +3194,19 @@
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3225,7 +3221,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3242,19 +3238,19 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3269,7 +3265,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3286,19 +3282,19 @@
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3313,7 +3309,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3330,19 +3326,19 @@
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3357,7 +3353,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3374,39 +3370,39 @@
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>DC Department of Human Resources</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3416,26 +3412,22 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
-        </is>
-      </c>
+      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Product Data Analyst, Servicing</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Upgrade, Inc.</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3445,7 +3437,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3463,29 +3455,29 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3503,74 +3495,82 @@
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr"/>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3578,27 +3578,23 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3630,19 +3626,19 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3657,7 +3653,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3674,19 +3670,19 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3701,7 +3697,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3718,19 +3714,19 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3745,7 +3741,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3762,24 +3758,24 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3789,7 +3785,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3806,24 +3802,24 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3833,7 +3829,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3850,19 +3846,19 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3877,7 +3873,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3899,14 +3895,14 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3943,14 +3939,14 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3987,19 +3983,19 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4009,7 +4005,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4026,19 +4022,19 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4053,7 +4049,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4075,19 +4071,19 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4097,7 +4093,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4114,19 +4110,19 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4141,7 +4137,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4158,19 +4154,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4185,7 +4181,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4202,19 +4198,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4229,7 +4225,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4246,19 +4242,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4273,7 +4269,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4290,19 +4286,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4334,19 +4330,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4361,7 +4357,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4378,19 +4374,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4405,7 +4401,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4427,14 +4423,14 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4449,7 +4445,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4466,19 +4462,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4493,7 +4489,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4510,19 +4506,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4537,7 +4533,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4554,19 +4550,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4581,7 +4577,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4598,19 +4594,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4625,7 +4621,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4642,19 +4638,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4669,7 +4665,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4691,7 +4687,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
         </is>
       </c>
     </row>
@@ -6723,8 +6719,44 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Business Analyst (Loyalty/Retention)</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Mercuryo</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>❓ Unknown</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Himalayas</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Hi! We're Mercuryo , and we're on a mission to redefine finance by blending the best of traditional banking with the power of decentralized finance (DeFi). We believe everyone deserves seamless access to Web3 and traditional financial services, so we're building the platform that makes it real: one that simplifies crypto and integrates it into the broader financial ecosystem. Since launching in 20</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J146"/>
+  <autoFilter ref="A1:J147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 09:09 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -5985,7 +5985,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6002,12 +6002,12 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 10:59 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -782,12 +782,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Principal Java Engineer II - Machine Learning - Elasticsearch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -807,26 +807,26 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -858,19 +858,19 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -902,19 +902,19 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -946,19 +946,19 @@
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -990,24 +990,24 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1034,24 +1034,24 @@
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Product (Crypto)</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1078,24 +1078,24 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Staff Data Scientist, Product (Crypto)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Menlo Park, CA; New York, NY</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1122,19 +1122,19 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1171,14 +1171,14 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
+          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1215,19 +1215,19 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1254,19 +1254,19 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1298,19 +1298,19 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1342,19 +1342,19 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1386,39 +1386,39 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SS&amp;C Technologies</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1428,22 +1428,26 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst - Junior</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Global Technical Talent, an Inc. 5000 Company</t>
+          <t>SS&amp;C Technologies</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1453,7 +1457,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Framingham, MA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1471,19 +1475,19 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Data Analyst - Junior</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SeatGeek</t>
+          <t>Global Technical Talent, an Inc. 5000 Company</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1493,7 +1497,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Framingham, MA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1511,7 +1515,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1527,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Betterment</t>
+          <t>SeatGeek</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1551,19 +1555,19 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Junior Data Scientist</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Betterment</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1573,7 +1577,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Texas, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1591,19 +1595,19 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Junior Data Scientist</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>Tech Consulting</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1613,7 +1617,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>Texas, United States</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1631,19 +1635,19 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>Brain Co.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1653,7 +1657,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco Bay Area</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1671,19 +1675,19 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4396367708</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst (Power BI)</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Chadwell Supply</t>
+          <t>SS&amp;C Technologies</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1693,7 +1697,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Florida, United States</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1711,19 +1715,19 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-ss-c-technologies-4386972427</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>University of Iowa</t>
+          <t>ATC</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1733,7 +1737,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Iowa City, IA</t>
+          <t>California, United States</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1751,19 +1755,19 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-atc-4395991558</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
+          <t>Value-Based Performance Reporting Analyst</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>DataAnnotation</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1773,7 +1777,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>Tennessee, United States</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1791,19 +1795,19 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
+          <t>https://www.linkedin.com/jobs/view/value-based-performance-reporting-analyst-at-dataannotation-4377566356</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I</t>
+          <t>Business Data Analyst I/II/Sr</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>RemoteHunter</t>
+          <t>Constellation</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1813,7 +1817,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Hurstbourne Acres, KY</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1831,19 +1835,19 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-at-remotehunter-4395975249</t>
+          <t>https://www.linkedin.com/jobs/view/business-data-analyst-i-ii-sr-at-constellation-4396333670</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Join Expert Network: Business Intelligence Analysts (Train AI Models Part Time!)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>MES Life Safety</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1853,7 +1857,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Sandy Hook, CT</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1871,19 +1875,19 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-mes-life-safety-4399227285</t>
+          <t>https://www.linkedin.com/jobs/view/join-expert-network-business-intelligence-analysts-train-ai-models-part-time%21-at-hackajob-4380450430</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Business Analyst - Private Capital</t>
+          <t>Performance Marketing Analyst, Paid Social &amp; Display</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1893,7 +1897,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1911,63 +1915,59 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
+          <t>https://www.linkedin.com/jobs/view/performance-marketing-analyst-paid-social-display-at-etsy-4399456051</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Highmark Residential</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Addison, TX</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-highmark-residential-4399405063</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1977,56 +1977,52 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>IMA Financial Group, Inc.</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2036,37 +2032,41 @@
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
+          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Entry Level Data Analyst</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2076,10 +2076,14 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2095,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Webologix Ltd/ INC</t>
+          <t>IMA Financial Group, Inc.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2101,7 +2105,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2119,19 +2123,19 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Entry Level Data Analyst</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>HirePower Staffing Solution</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2141,7 +2145,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Fullerton, CA</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2159,19 +2163,19 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Entry Level Machine Learning Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>Webologix Ltd/ INC</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2181,7 +2185,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2199,19 +2203,19 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>HirePower Staffing Solution</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2221,7 +2225,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Fullerton, CA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2239,19 +2243,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CCAR Business Analyst</t>
+          <t>Entry Level Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mitchell Martin Inc.</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2261,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Jersey City, NJ</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2279,19 +2283,19 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>CCAR Business Analyst</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Aditi Consulting</t>
+          <t>Mitchell Martin Inc.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2301,7 +2305,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Chillicothe, IL</t>
+          <t>Jersey City, NJ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2319,7 +2323,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
+          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2410,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst, Digital Media</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Taboola</t>
+          <t>Aditi Consulting</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2421,7 +2425,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chillicothe, IL</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2439,63 +2443,59 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-digital-media-at-taboola-4398368627</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Meet Life Sciences</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2522,19 +2522,19 @@
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2571,34 +2571,34 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2608,22 +2608,26 @@
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2633,7 +2637,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2651,19 +2655,19 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>FNS, Inc.</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2673,7 +2677,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2691,7 +2695,7 @@
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-fns-inc-4385265212</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2910,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2921,7 +2925,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2938,19 +2942,19 @@
       <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2965,7 +2969,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2987,14 +2991,14 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3009,7 +3013,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3031,34 +3035,34 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Data &amp; Business Intelligence Analyst</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3068,22 +3072,26 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>BI Data Analyst</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Uline</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3093,7 +3101,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Cedar Rapids, IA</t>
+          <t>Milwaukee, WI</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3111,7 +3119,7 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-uline-4383941437</t>
         </is>
       </c>
     </row>
@@ -3502,12 +3510,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Robert Half</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3517,104 +3525,92 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
-        </is>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-robert-half-4395319491</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Dynasticx LLC</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>New Jersey, United States</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
-        </is>
-      </c>
+      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-dynasticx-llc-4395364932</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3622,23 +3618,27 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3670,19 +3670,19 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3714,19 +3714,19 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3758,24 +3758,24 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3802,24 +3802,24 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3846,24 +3846,24 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3890,19 +3890,19 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3939,14 +3939,14 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3983,19 +3983,19 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4022,24 +4022,24 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4066,24 +4066,24 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4110,24 +4110,24 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4154,19 +4154,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4198,19 +4198,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4242,19 +4242,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4286,19 +4286,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4335,14 +4335,14 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4357,7 +4357,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4374,19 +4374,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4401,7 +4401,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4418,19 +4418,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4462,19 +4462,19 @@
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4506,19 +4506,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4550,19 +4550,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4577,7 +4577,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4594,19 +4594,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4638,19 +4638,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4682,19 +4682,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7376835</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4709,7 +4709,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4726,19 +4726,19 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4770,34 +4770,34 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Tempe, Arizona, United States</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4807,26 +4807,26 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594392?gh_jid=7594392</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -4858,19 +4858,19 @@
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594416?gh_jid=7594416</t>
+          <t>http://www.hioscar.com/careers/7594392?gh_jid=7594392</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Tempe, Arizona, United States</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4902,19 +4902,19 @@
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7594416?gh_jid=7594416</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -4946,19 +4946,19 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4995,29 +4995,29 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5027,26 +5027,26 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5078,19 +5078,19 @@
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5122,24 +5122,24 @@
       <c r="H110" s="2" t="inlineStr"/>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5149,7 +5149,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5159,31 +5159,31 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -5203,26 +5203,26 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5259,19 +5259,19 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5291,31 +5291,31 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5335,26 +5335,26 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5391,29 +5391,29 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5423,41 +5423,41 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Principal Software Engineer II - Machine Learning - Elasticsearch</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5467,19 +5467,19 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735255&amp;gh_jid=7735255</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
@@ -5985,7 +5985,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6002,12 +6002,12 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
+          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 13:27 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -797,7 +797,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -819,239 +819,219 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Junior AI/ML Engineer (Data &amp; Cloud Platforms)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Mod Op</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.linkedin.com/jobs/view/junior-ai-ml-engineer-data-cloud-platforms-at-mod-op-4399859352</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384795150</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>ML Engineer</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Catalyst Labs</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.linkedin.com/jobs/view/ml-engineer-at-catalyst-labs-4398673366</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Junior Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Emerald Resource Group</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Broadview Heights, OH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
-        </is>
-      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.linkedin.com/jobs/view/junior-business-intelligence-analyst-at-emerald-resource-group-4400208330</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Data Analyst - Power BI Dashboard Development</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Accylerate</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
-        </is>
-      </c>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-power-bi-dashboard-development-at-accylerate-4399855505</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1061,7 +1041,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1078,24 +1058,24 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Product (Crypto)</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1105,7 +1085,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1122,24 +1102,24 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1149,7 +1129,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1166,24 +1146,24 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1193,7 +1173,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1210,24 +1190,24 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1237,7 +1217,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1254,24 +1234,24 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1281,7 +1261,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1298,24 +1278,24 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Staff Data Scientist, Product (Crypto)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1325,7 +1305,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Menlo Park, CA; New York, NY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1342,24 +1322,24 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1369,7 +1349,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1386,24 +1366,24 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1413,7 +1393,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1430,39 +1410,39 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>SS&amp;C Technologies</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1472,37 +1452,41 @@
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Data Analyst - Junior</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Global Technical Talent, an Inc. 5000 Company</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Framingham, MA</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1512,37 +1496,41 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>SeatGeek</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1552,37 +1540,41 @@
       </c>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Betterment</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1592,37 +1584,41 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Junior Data Scientist</t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Tech Consulting</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Texas, United States</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1632,22 +1628,26 @@
       </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-data-scientist-at-tech-consulting-4395975986</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>SS&amp;C Technologies</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1675,19 +1675,19 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst - Junior</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>SS&amp;C Technologies</t>
+          <t>Global Technical Talent, an Inc. 5000 Company</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Florida, United States</t>
+          <t>Framingham, MA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1715,19 +1715,19 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-ss-c-technologies-4386972427</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ATC</t>
+          <t>SeatGeek</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>California, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1755,19 +1755,19 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-atc-4395991558</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Value-Based Performance Reporting Analyst</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>DataAnnotation</t>
+          <t>Betterment</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Tennessee, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1795,19 +1795,19 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/value-based-performance-reporting-analyst-at-dataannotation-4377566356</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Business Data Analyst I/II/Sr</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Constellation</t>
+          <t>Brain Co.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Hurstbourne Acres, KY</t>
+          <t>San Francisco Bay Area</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1835,19 +1835,19 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-data-analyst-i-ii-sr-at-constellation-4396333670</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Join Expert Network: Business Intelligence Analysts (Train AI Models Part Time!)</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1875,29 +1875,29 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/join-expert-network-business-intelligence-analysts-train-ai-models-part-time%21-at-hackajob-4380450430</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4396367708</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Performance Marketing Analyst, Paid Social &amp; Display</t>
+          <t>Business Intelligence Analyst (Power BI)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Chadwell Supply</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1915,7 +1915,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/performance-marketing-analyst-paid-social-display-at-etsy-4399456051</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Highmark Residential</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Addison, TX</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1955,29 +1955,29 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-highmark-residential-4399405063</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Business Analyst - Private Capital</t>
+          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1995,19 +1995,19 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2017,100 +2017,92 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>LSC - LifeSciences Consultants</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4399271713</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>IMA Financial Group, Inc.</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2120,37 +2112,41 @@
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
+          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Entry Level Data Analyst</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2160,10 +2156,14 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Webologix Ltd/ INC</t>
+          <t>IMA Financial Group, Inc.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2203,19 +2203,19 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Entry Level Data Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>HirePower Staffing Solution</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Fullerton, CA</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,19 +2243,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Entry Level Machine Learning Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>Webologix Ltd/ INC</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,19 +2283,19 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CCAR Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mitchell Martin Inc.</t>
+          <t>HirePower Staffing Solution</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Jersey City, NJ</t>
+          <t>Fullerton, CA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,19 +2323,19 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Entry Level Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2363,19 +2363,19 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Greater Chicago Area</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2403,19 +2403,19 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>CCAR Business Analyst</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Aditi Consulting</t>
+          <t>Mitchell Martin Inc.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Chillicothe, IL</t>
+          <t>Jersey City, NJ</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2443,19 +2443,19 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
+          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Meet Life Sciences</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2483,107 +2483,99 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-meet-life-sciences-4398414637</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Greater Chicago Area</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Aditi Consulting</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Chillicothe, IL</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2593,7 +2585,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2610,39 +2602,39 @@
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2652,37 +2644,41 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2692,22 +2688,26 @@
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Empower</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -2735,19 +2735,19 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Lucid Software</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
@@ -2775,29 +2775,29 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Data Scientist, Customer Support Analytics</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Empower</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
@@ -2815,63 +2815,59 @@
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-empower-4382065637</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Lucid Software</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
-        </is>
-      </c>
+      <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-lucid-software-4397353420</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Inference, Global Markets</t>
+          <t>Data Scientist, Customer Support Analytics</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2881,41 +2877,37 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
-        </is>
-      </c>
+      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-customer-support-analytics-at-etsy-4397396983</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2925,7 +2917,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2942,24 +2934,24 @@
       <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5115935008</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Senior Data Scientist - Inference, Global Markets</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2969,7 +2961,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2986,24 +2978,24 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://careers.airbnb.com/positions/7446449?gh_jid=7446449</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Software Engineer, Machine Learning Infrastructure</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3013,7 +3005,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Seattle, San Francisco</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3030,19 +3022,19 @@
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3057,7 +3049,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3079,34 +3071,34 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Uline</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Milwaukee, WI</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3116,22 +3108,26 @@
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-uline-4383941437</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Trust</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3141,7 +3137,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3151,163 +3147,151 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager, Product</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
-        </is>
-      </c>
+      <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>People Operations Analyst</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
-        </is>
-      </c>
+      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795052</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Senior Product Data Scientist (Analyst)</t>
+          <t>BI Data Analyst</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Warsaw</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
-        </is>
-      </c>
+      <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
+          <t>https://www.linkedin.com/jobs/view/bi-data-analyst-at-motion-4332095380</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Senior Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Asana</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3317,7 +3301,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3334,19 +3318,19 @@
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
+          <t>https://careers.airbnb.com/positions/7700249?gh_jid=7700249</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Marketing</t>
+          <t>Data Science Manager, Product</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3378,39 +3362,39 @@
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Product Data Science team, you will be a key player in using data and scientific techniques to inform Asana’s product strategy and make product decisions. You will work closely with Engineering, Product, and Design</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
+          <t>https://www.asana.com/jobs/apply/7584394?gh_jid=7584394</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>People Operations Analyst</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>DC Department of Human Resources</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3420,37 +3404,41 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The People Team is a global team responsible for helping Asana scale with clarity, focus, and impact. We partner closely with leaders across the company to enable performance, develop talent, and build systems that support strong execution and a great employee experience. Our work spans talent and performance management, rewards, employee relations, people partnerships, and people analyti</t>
+        </is>
+      </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-dc-department-of-human-resources-4395297713</t>
+          <t>https://www.asana.com/jobs/apply/7657532?gh_jid=7657532</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Product Data Analyst, Servicing</t>
+          <t>Senior Product Data Scientist (Analyst)</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Upgrade, Inc.</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Warsaw</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3460,22 +3448,26 @@
       </c>
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: arial, helvetica, sans-serif;&amp;quot;&amp;gt;Asanas &amp;lt;strong&amp;gt;Data Science&amp;lt;/strong&amp;gt; team helps us fulfill our mission by informing strategy, defining success metrics, and identifying new ways to deliver user value. Data scientists are at the crux of deepening our understanding of the customers and driving more business outcomes by leveraging experimen</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/product-data-analyst-servicing-at-upgrade-inc-4321559093</t>
+          <t>https://www.asana.com/jobs/apply/6352958?gh_jid=6352958</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3485,12 +3477,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3500,37 +3492,41 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Were looking for a Staff Data Scientist to help define Asanas growth strategy as users increasingly discover and adopt software through LLM interfaces like ChatGPT, Claude, and Gemini. With millions of knowledge workers now starting their workday in conversational AI tools, were at an inflection point in how productivity software reaches users. Youll drive Asanas acquisition playbook for </t>
+        </is>
+      </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://www.asana.com/jobs/apply/7555480?gh_jid=7555480</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Staff Data Scientist, Marketing</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Robert Half</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3540,32 +3536,36 @@
       </c>
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;p&amp;gt;The Data Science team at Asana is pivotal in fulfilling our mission by fostering a data-driven approach in shaping both our product and business strategies. In your role on the Marketing Data Science team, you will be the deepest technical expert responsible for using data and scientific techniques to design and build scalable, state-of-the-art solutions to enhance Asana’s marketing effec</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-robert-half-4395319491</t>
+          <t>https://www.asana.com/jobs/apply/7612064?gh_jid=7612064</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Scientist - Campus Full-Time</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dynasticx LLC</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>New Jersey, United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3583,7 +3583,7 @@
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-dynasticx-llc-4395364932</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexico City </t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4286,12 +4286,12 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
         </is>
       </c>
     </row>
@@ -5985,7 +5985,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6002,12 +6002,12 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p data-renderer-start-pos=&amp;quot;1648&amp;quot;&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges </t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7641390002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 15:24 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$145</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -797,7 +797,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7440363&amp;gh_jid=7440363</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7735254&amp;gh_jid=7735254</t>
         </is>
       </c>
     </row>
@@ -866,17 +866,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Data Scientist, All Levels</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Oscar Health</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -899,19 +899,19 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384795150</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4387600293</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ML Engineer</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Catalyst Labs</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -939,19 +939,19 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ml-engineer-at-catalyst-labs-4398673366</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384795150</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Junior Business Intelligence Analyst</t>
+          <t>ML Engineer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Emerald Resource Group</t>
+          <t>Catalyst Labs</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Broadview Heights, OH</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -979,19 +979,19 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-business-intelligence-analyst-at-emerald-resource-group-4400208330</t>
+          <t>https://www.linkedin.com/jobs/view/ml-engineer-at-catalyst-labs-4398673366</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst - Power BI Dashboard Development</t>
+          <t>Junior Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Accylerate</t>
+          <t>Emerald Resource Group</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Broadview Heights, OH</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1019,58 +1019,54 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-power-bi-dashboard-development-at-accylerate-4399855505</t>
+          <t>https://www.linkedin.com/jobs/view/junior-business-intelligence-analyst-at-emerald-resource-group-4400208330</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Data Analyst - Power BI Dashboard Development</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Accylerate</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-power-bi-dashboard-development-at-accylerate-4399855505</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1085,7 +1081,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1102,19 +1098,19 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1129,7 +1125,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1146,19 +1142,19 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1190,19 +1186,19 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1217,7 +1213,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1234,24 +1230,24 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1261,7 +1257,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1278,24 +1274,24 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Product (Crypto)</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1305,7 +1301,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1322,24 +1318,24 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Staff Data Scientist, Product (Crypto)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1349,7 +1345,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Menlo Park, CA; New York, NY</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1366,19 +1362,19 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1393,7 +1389,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1415,14 +1411,14 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
+          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1437,7 +1433,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1459,19 +1455,19 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1481,7 +1477,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1498,19 +1494,19 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1525,7 +1521,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1542,19 +1538,19 @@
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1569,7 +1565,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1586,19 +1582,19 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1613,7 +1609,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1630,39 +1626,39 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SS&amp;C Technologies</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1672,22 +1668,26 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst - Junior</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global Technical Talent, an Inc. 5000 Company</t>
+          <t>SS&amp;C Technologies</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Framingham, MA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1715,19 +1715,19 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Data Analyst - Junior</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SeatGeek</t>
+          <t>Global Technical Talent, an Inc. 5000 Company</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Framingham, MA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1755,7 +1755,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Betterment</t>
+          <t>SeatGeek</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1795,19 +1795,19 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>Betterment</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1835,19 +1835,19 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>AI/ML Engineer</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>Brain Co.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>San Francisco Bay Area</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1875,19 +1875,19 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4396367708</t>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst (Power BI)</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Chadwell Supply</t>
+          <t>Optum</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1915,19 +1915,19 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-optum-4396367708</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst</t>
+          <t>Business Intelligence Analyst (Power BI)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>University of Iowa</t>
+          <t>Chadwell Supply</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Iowa City, IA</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1955,19 +1955,19 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-power-bi-at-chadwell-supply-4395995721</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
+          <t>Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Unum</t>
+          <t>University of Iowa</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Chattanooga, TN</t>
+          <t>Iowa City, IA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1995,29 +1995,29 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-at-university-of-iowa-4395923318</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst - Private Capital</t>
+          <t>Business Intelligence Analyst I - Tableau/Excel/Salesforce proficiency</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Unum</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chattanooga, TN</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2035,29 +2035,29 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-analyst-i-tableau-excel-salesforce-proficiency-at-unum-4384752636</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
+          <t>Business Analyst - Private Capital</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LSC - LifeSciences Consultants</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2075,7 +2075,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4399271713</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-private-capital-at-mckinsey-company-4386789481</t>
         </is>
       </c>
     </row>
@@ -2450,12 +2450,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Greater Chicago Area</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2483,19 +2483,19 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Greater Chicago Area</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2523,7 +2523,7 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
@@ -2570,56 +2570,52 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Supportability</t>
+          <t>Business Analyst, Digital Media</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Taboola</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
-        </is>
-      </c>
+      <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-digital-media-at-taboola-4398368627</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
+          <t>Machine Learning Engineer, Supportability</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2629,7 +2625,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2646,19 +2642,19 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7384709</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Agentic</t>
+          <t xml:space="preserve">Senior Data Scientist, Fraud </t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2673,7 +2669,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2695,34 +2691,34 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7412037?t=gh_src=&amp;gh_jid=7412037</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>M Science</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>New York City Metropolitan Area</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2732,22 +2728,26 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+        </is>
+      </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7676714?t=gh_src=&amp;gh_jid=7676714</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>M Science</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City Metropolitan Area</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2775,7 +2775,7 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-hackajob-4382830392</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-m-science-4394480305</t>
         </is>
       </c>
     </row>
@@ -3550,67 +3550,75 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Data Scientist - Campus Full-Time</t>
+          <t>Payments &amp;amp; Billing Operations Analyst</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Automatiq</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>New York, United States</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr"/>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>analyst, salesforce, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
+        </is>
+      </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-campus-full-time-at-two-sigma-4351354278</t>
+          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Payments &amp;amp; Billing Operations Analyst</t>
+          <t>GTM Strategy and Operations Analyst - EMEA</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Automatiq</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3618,27 +3626,23 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>analyst, salesforce, system, training, technical, support</t>
-        </is>
-      </c>
+      <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>The Payments &amp; Billing Operations Analyst plays a key role in managing billing operations, collections, supporting payments processes, and mitigating payment-related discrepancies all while maintaining excellent customer service and compliance with operational standards. The role is a part of the finance team, reporting to the Billing and Collections Manager and involves collaboration with multipl</t>
+          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-payments-amp-billing-operations-analyst-automatiq-1130956</t>
+          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GTM Strategy and Operations Analyst - EMEA</t>
+          <t>Order Operations Analyst (Dublin)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3670,19 +3674,19 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;About the Role&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Datadog’s GTM Strategy &amp;amp; Operations team runs the business at scale. We ensure our sales engine operates cleanly, fairly, and efficiently while continuously improving how we drive growth.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;This Analyst role is foundational to EMEA performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;You will own the operational integrity of our sales motion - clean boo</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7636353/?gh_jid=7636353</t>
+          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Order Operations Analyst (Dublin)</t>
+          <t>Senior Applied Scientist</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3697,7 +3701,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3714,19 +3718,19 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Order Operations Analyst&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;We are looking for an Order Operations Analyst to join our evolving Sales Operations team located in our Dublin office. The ideal candidate thrives in high-growth, collaborative environments and is eager to dive into the Order Operations function of the Sales process. We need a detail-oriented, process-minded individ</t>
+          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7585493/?gh_jid=7585493</t>
+          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist</t>
+          <t>Senior People Analyst</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3741,7 +3745,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>New York, New York, USA</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3758,19 +3762,19 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The Applied AI team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;anomaly detection&amp;lt;/a&amp;gt;, &amp;lt;a href=&amp;quot;https://docs.datadoghq.com/logs/explorer/watchdog_insights/&amp;quot;&amp;gt;error outliers&amp;lt;/a&amp;</t>
+          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/6781197/?gh_jid=6781197</t>
+          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Senior People Analyst</t>
+          <t>Senior Software Engineer - Data Science</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3785,7 +3789,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, USA</t>
+          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3802,24 +3806,24 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The People Analytics Team at Datadog uses data to help our growing organization make better people decisions. In this role, you’ll partner with People and business leadership to deliver analyses, dashboards, and insights that shape how we hire, develop, retain, and support Datadogs across the world.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;em&amp;gt;At Datadog, we place value in our office culture—the re</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7493743/?gh_jid=7493743</t>
+          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Science</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Datadog</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3829,7 +3833,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Bordeaux, France; Grenoble, France; Lyon, France; Madrid, Spain; Montpellier, France; Nantes, France; Paris, France; Sophia Antipolis, France</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3846,24 +3850,24 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;The Data Science team designs and builds algorithmically driven features in the Datadog app. We work across a range of applications, primarily focusing on analysis on streaming data such as &amp;lt;/span&amp;gt;&amp;lt;a href=&amp;quot;https://www.datadoghq.com/blog/watchdog/&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;anomaly detection&amp;lt;/spa</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://careers.datadoghq.com/detail/7472886/?gh_jid=7472886</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Data Analyst</t>
+          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3873,7 +3877,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3890,19 +3894,19 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Data Science Engineer, Capacity &amp; Efficiency</t>
+          <t>Machine Learning Systems Engineer, Research Tools</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3917,7 +3921,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>New York City, NY; San Francisco, CA | New York City, NY; Seattle, WA</t>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3939,14 +3943,14 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5125881008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, Research Tools</t>
+          <t>Machine Learning Systems Engineer, RL Engineering</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3983,14 +3987,14 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952079008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer, RL Engineering</t>
+          <t>Support Operations Analyst</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4027,19 +4031,19 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Support Operations Analyst</t>
+          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4049,7 +4053,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4066,19 +4070,19 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Anthropic&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Anthropic’s mission is to create reliable, interpretable, and steerable AI systems. We want AI to be safe and beneficial for our users and for society as a whole. Our team is a quickly growing group of committed researchers, engineers, policy experts, and business leaders working t</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5080931008</t>
+          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Senior/ Manager, Machine Learning, Community Support Products</t>
+          <t xml:space="preserve">Staff Analytics Engineer </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4093,7 +4097,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4115,19 +4119,19 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7672101?gh_jid=7672101</t>
+          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Analytics Engineer </t>
+          <t>AI/ML Engineering Manager, Payment Intelligence</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4137,7 +4141,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>US-SF, US-NYC, US-SEA</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4154,19 +4158,19 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7733495?gh_jid=7733495</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>AI/ML Engineering Manager, Payment Intelligence</t>
+          <t>Credit Operations Analyst</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4181,7 +4185,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>US-SF, US-NYC, US-SEA</t>
+          <t>Chicago, Toronto, US-Remote</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4198,19 +4202,19 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe’s mission is to accelerate global economic and technological development. We offer financial infrastructure and a variety of services to serve the needs of a wide range of users, from startups to enterprises, with global scale and industry-leading reliability and product quality.&amp;nbsp; All financial services business</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7286376</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Credit Operations Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4225,7 +4229,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Chicago, Toronto, US-Remote</t>
+          <t xml:space="preserve">Mexico City </t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4242,19 +4246,19 @@
       <c r="H90" s="2" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7722938</t>
+          <t>https://stripe.com/jobs/search?gh_jid=6282403</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data Science Manager</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4269,7 +4273,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Seattle, WA OR New York, NY OR Remote North America</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4286,19 +4290,19 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering amoun</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5416444</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Data Science Manager</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4313,7 +4317,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA OR New York, NY OR Remote North America</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4330,19 +4334,19 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7644403</t>
+          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Engineering Manager, Machine Learning Platform</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4374,19 +4378,19 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line g</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=5895430</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Engineering Manager, Machine Learning Platform</t>
+          <t>Financial Data Analyst, SDC</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4401,7 +4405,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4418,19 +4422,19 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7712852</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, SDC</t>
+          <t>Financial Data Analyst, Technical Operations</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4445,7 +4449,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Dublin, Ireland</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4467,14 +4471,14 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7525640</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Financial Data Analyst, Technical Operations</t>
+          <t>Financial Data Analyst-User Billing</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4489,7 +4493,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4506,19 +4510,19 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7061516</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Financial Data Analyst-User Billing</t>
+          <t>Machine Learning Engineer, Payments ML Accelerator</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4533,7 +4537,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Seattle; San Francisco; New York City</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4550,19 +4554,19 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to</t>
+          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7278434</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Payments ML Accelerator</t>
+          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4577,7 +4581,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City</t>
+          <t>Seattle; San Francisco; New York City; Remote</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4594,19 +4598,19 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payment</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7079044</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine Learning Engineer, Stripe Assistant </t>
+          <t>PhD Machine Learning Engineer, New Grad</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4621,7 +4625,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Seattle; San Francisco; New York City; Remote</t>
+          <t>San Francisco, New York City, Seattle</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4638,19 +4642,19 @@
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to inc</t>
+          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7629052</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>PhD Machine Learning Engineer, New Grad</t>
+          <t>Risk Operations Analyst, Financial Crimes</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4665,7 +4669,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, New York City, Seattle</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4682,19 +4686,19 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the GDP of the internet, and we have a staggering am</t>
+          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7216668</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Risk Operations Analyst, Financial Crimes</t>
+          <t>Staff Data Scientist</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4709,7 +4713,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4726,19 +4730,19 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7430332</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist</t>
+          <t>Strategy &amp; Operations Analyst, Customer Success</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4753,7 +4757,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t xml:space="preserve">Chicago </t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4770,34 +4774,34 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;ace-line gutter-author-p-118095 emptyGutter&amp;quot;&amp;gt; &amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7568328</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Analyst, Customer Success</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chicago </t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4807,26 +4811,26 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;Who we are &amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About Stripe&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies - from the world’s largest enterprises to the most ambitious startups - use Stripe to accept payments, grow their revenue, and acceler</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7397878</t>
+          <t>http://www.hioscar.com/careers/7592274?gh_jid=7592274</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Data Scientist II</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -4841,7 +4845,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Tempe, Arizona, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4858,19 +4862,19 @@
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist I to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;g</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594392?gh_jid=7594392</t>
+          <t>http://www.hioscar.com/careers/7592301?gh_jid=7592301</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Data Scientist II</t>
+          <t>Senior Data Scientist, Advanced Risk Modeling</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4885,7 +4889,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Tempe, Arizona, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4902,19 +4906,19 @@
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Data Scientist II to join our Data team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves - one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;p&amp;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7594416?gh_jid=7594416</t>
+          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Advanced Risk Modeling</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4929,7 +4933,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>Los Angeles, California, United States</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -4946,19 +4950,19 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Data Team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a relentless focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;</t>
+          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7373481?gh_jid=7373481</t>
+          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior</t>
+          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4973,7 +4977,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Los Angeles, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4995,29 +4999,29 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7592191?gh_jid=7592191</t>
+          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Data &amp; Member Behavior (Campaign Optimization)</t>
+          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>New York, New York, United States</t>
+          <t>San Francisco, CA; Austin, TX; New York, NY</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5027,26 +5031,26 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;Hi, were Oscar. Were hiring a Senior Data Scientist to join our Engineering team.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Oscar is the first health insurance company built around a full stack technology platform and a focus on serving our members. We started Oscar in 2012 to create the kind of health insurance company we would want for ourselves—one that behaves like a doctor in the family.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;g</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>http://www.hioscar.com/careers/7268251?gh_jid=7268251</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (AI &amp; Analytics Platform)</t>
+          <t>AI Analytics Engineer (Business Analytics)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5078,19 +5082,19 @@
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable is building the infrastructure that makes AI-powered analyti</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434287002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Business Analytics)</t>
+          <t>AI Analytics Engineer (Marketing Analytics)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5122,24 +5126,24 @@
       <c r="H110" s="2" t="inlineStr"/>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Join Airtable as an &amp;lt;strong&amp;gt;Analytics Engineer&amp;lt;/strong&amp;gt; s</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8470036002</t>
+          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AI Analytics Engineer (Marketing Analytics)</t>
+          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Airtable</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5149,7 +5153,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>San Francisco, CA; Austin, TX; New York, NY</t>
+          <t>New York; San Francisco, California</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5159,31 +5163,31 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Airtable is the no-code app platform that empowers people closest to the work to accelerate their most critical business processes. More than 500,000 organizations, including 80% of the Fortune 100, rely on Airtable to transform how work gets done.&amp;lt;/p&amp;gt;&amp;lt;/div&amp;gt;&amp;lt;p&amp;gt;Airtable’s Data Science &amp;amp; Analytics team seeks an Analytics Engin</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/airtable/jobs/8434307002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Sr Analytics Engineer - GTM Strategy and Operations</t>
+          <t>Senior Business Analyst, Brazil</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -5193,7 +5197,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>New York; San Francisco, California</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -5203,26 +5207,26 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;SLSQ227R554&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 10pt;&amp;quot;&amp;gt;&amp;lt;strong&amp;gt;Sr Analytics Engineer - GTM Strategy and Operations&amp;lt;/strong&amp;gt;&amp;lt;/span&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8479036002</t>
+          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Brazil</t>
+          <t>Senior Business Analyst, Mexico</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5237,7 +5241,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5259,19 +5263,19 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7758637?gh_jid=7758637</t>
+          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Mexico</t>
+          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Elastic</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -5281,7 +5285,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Barcelona, Spain</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5291,31 +5295,31 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7669533?gh_jid=7669533</t>
+          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Senior Data Analyst – Insights &amp; Analytics (Revenue Operations)</t>
+          <t>Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Elastic</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5325,7 +5329,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Barcelona, Spain</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5335,26 +5339,26 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Elastic, the Search AI Company, enables everyone to find the answers they need in real time, using all their data, at scale — unleashing the potential of businesses and people. The Elastic Search AI Platform, used by more than 50% of the Fortune 500, brings together the precision of search and the intelligence of AI to enable everyone to accelera</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=7601880&amp;gh_jid=7601880</t>
+          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, Community Support Engineering</t>
+          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5391,29 +5395,29 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7716341?gh_jid=7716341</t>
+          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Senior/Staff Machine Learning Engineer, Community Support Engineering</t>
+          <t>People Analytics &amp; Insights Analyst</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Argentina Remote</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5423,41 +5427,41 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7693033?gh_jid=7693033</t>
+          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>People Analytics &amp; Insights Analyst</t>
+          <t>Senior Data Analyst, Trust &amp; Safety</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Argentina Remote</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5467,31 +5471,31 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;At Webflow, we’re building the world’s leading AI-native Digital Experience Platform, and we’re doing it as a remote-first company built on trust, transparency, and a whole lot of creativity. This work takes grit, because we move fast, without ever sacrificing craft or quality. Our mission is to bring development superpowers to everyone. From entrepreneurs launching their first idea to gl</t>
+          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/webflow/jobs/7657237</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Trust &amp; Safety</t>
+          <t>Data Scientist, Product</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5501,7 +5505,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5511,26 +5515,26 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Trust &amp;amp; Safety Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build security awareness and adoption, keeping our members and Chime safe. Trust &amp;amp; Safety organization’s mission is to make Chime the most trusted financial partner by safeguardi</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344063002?gh_jid=8344063002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist, Product</t>
+          <t>Senior Analytics Engineer, Corporate Strategy</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -5545,7 +5549,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -5567,14 +5571,14 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324983?t=gh_src=&amp;gh_jid=7324983</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Senior Analytics Engineer, Corporate Strategy</t>
+          <t>Senior Data Scientist, Product</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5611,19 +5615,19 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7346630?t=gh_src=&amp;gh_jid=7346630</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, Product</t>
+          <t>Senior Data Analyst, Spending</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -5633,7 +5637,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5650,19 +5654,19 @@
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7324981?t=gh_src=&amp;gh_jid=7324981</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Senior Data Analyst, Spending</t>
+          <t>Sr. Data Analyst, Lifecycle Marketing</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5677,7 +5681,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5694,24 +5698,24 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a Spending Product Analyst, you will have the opportunity to develop, test, launch and scale member banking experience products that build products that make Chime banking the best place to spend, save and invest. Spending XFN organization’s mission is to deliver industry-leading spending products that members want to keep </t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8344077002?gh_jid=8344077002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst, Lifecycle Marketing</t>
+          <t xml:space="preserve">Staff Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -5721,7 +5725,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5731,26 +5735,26 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lifecycle Marketing Data Analyst to help us better understand how our members engage across the customer journey and how we use our owned channels to communicate with them, from onboarding to long-term retention. As our Lifecycle Marketing Data Analyst, you’ll partner closely with Lifecycle Marketing to report</t>
+          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8445046002?gh_jid=8445046002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Machine Learning Engineer </t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5765,7 +5769,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5775,31 +5779,31 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1504&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8401114002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t>Senior Staff Machine Learning Engineer, Trust</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -5809,7 +5813,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Remote - California; San Francisco, California; Seattle, Washington</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5819,26 +5823,26 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr"/>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ427R169&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;While candidates in the listed locations are encouraged for this role, we are open to remote candidates in other locations.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a &amp;lt;strong&amp;gt;Principal Data Scientist&amp;lt;/strong&amp;gt; to serve as the statistical voice of the Data Science organization. This person will make Databricks sm</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8456277002</t>
+          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Trust</t>
+          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5853,7 +5857,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5863,7 +5867,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
@@ -5875,14 +5879,14 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7592146?gh_jid=7592146</t>
+          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Data &amp; Eval</t>
+          <t>Staff Data Scientist, Forecasting-Finance</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -5897,7 +5901,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t xml:space="preserve">United States </t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5907,7 +5911,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr"/>
@@ -5919,19 +5923,19 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/6757302?gh_jid=6757302</t>
+          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Forecasting-Finance</t>
+          <t>Senior Manager, Infrastructure Data Science</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5941,7 +5945,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States </t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5951,26 +5955,26 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7551313?gh_jid=7551313</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Senior Manager, Infrastructure Data Science</t>
+          <t>Sr. Data Analyst</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5985,7 +5989,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6002,19 +6006,19 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p data-pm-slice=&amp;quot;1 1 []&amp;quot;&amp;gt;RDQ225R487&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;Job Description&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Databricks is looking for a Senior Manager, Infrastructure Data Science to shape the future of Databricks infrastructure through data science. You will tackle some of the most complex challenges related to capacity planning, performance optimization, reliability</t>
+          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7734812002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Sr. Data Analyst</t>
+          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -6029,7 +6033,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6039,26 +6043,26 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h5&amp;gt;&amp;lt;strong&amp;gt;Req ID: GAQ126R127&amp;lt;/strong&amp;gt;&amp;lt;/h5&amp;gt; &amp;lt;h5&amp;gt;The Sr. Data Analyst (Tableau) is key in technological decision-making for business teams’ future data, analysis, and reporting needs. The role supports the business’s daily operations, including troubleshooting the data intelligence warehouse environment and monitoring jobs. It is also the role of the analyst to guide </t>
+          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7808221002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Machine Learning Engineer - GenAI Platform </t>
+          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6090,19 +6094,19 @@
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-984&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in late 2020 by a small group of machine learning engineers and researchers, Mosaic AI enables companies to securely fine-tune, train and deploy custom AI models on their own data, for maximum security and control. Compatible with all major cloud providers, the Mosaic AI platform provides maximum flexibility for AI development. Introduced in 2023, Mosaic A</t>
+          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=6954585002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Machine Learning Engineer </t>
+          <t xml:space="preserve">Staff Data Scientist </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6134,19 +6138,19 @@
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1131&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing GenAI-powered products. Over the past years, we’ve launched&amp;nbsp;&amp;lt;a class=&amp;quot;c-link&amp;quot; href=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;quot; target=&amp;quot;_blank&amp;quot; data-stringify-link=&amp;quot;https://www.databricks.com/blog/introducing-databricks-assistant&amp;q</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7276195002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data Scientist </t>
+          <t>Staff Data Scientist - Infrastructure</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -6161,7 +6165,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Mountain View, California</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6178,19 +6182,19 @@
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems, from security threat detection to cancer drug development. We do this by building and running the worlds best Data Intelligence Platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by </t>
+          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=5507088002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Staff Data Scientist - Infrastructure</t>
+          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6205,7 +6209,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Mountain View, California</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6222,19 +6226,19 @@
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-57&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;At Databricks, we are obsessed with enabling data teams to solve the worlds toughest problems. We do this by building and running the worlds best data and AI infrastructure platform, so our customers can focus on the high value challenges that are central to their own missions.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Founded in 2013 by the original creators of</t>
+          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7069793002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Staff Data Scientist - Trust and Safety</t>
+          <t>Staff Software Engineer - Machine Learning (Search)</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6249,7 +6253,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6266,24 +6270,24 @@
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;RDQ426R282&amp;lt;br&amp;gt;&amp;lt;br&amp;gt;Databricks is building the worlds best and most secure platform for data and AI. We innovate and deploy industry-leading solutions in security, compliance, and governance.&amp;nbsp;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;As a member of the Trust and Safety Data Science team, you will work on projects critical to ensuring the security and compliance of the Databricks Platform. Our cu</t>
+          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=8178287002</t>
+          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Machine Learning (Search)</t>
+          <t>HR Analyst</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>SurveyMonkey</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6293,99 +6297,99 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="G137" t="inlineStr"/>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>hr, analyst, system, training, technical, support</t>
+        </is>
+      </c>
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;P-1408&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;The Applied AI team at Databricks sits at the forefront of advancing AI/ML-powered products&amp;lt;/strong&amp;gt;. Databricks’ customers are continuously creating new assets (tables, notebooks, dashboards, datarooms, pipelines, sql queries, ml models etc.) on the platform. Some of them can have hundreds of millions of assets. Finding an asset is a critical</t>
+          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://databricks.com/company/careers/open-positions/job?gh_jid=7958982002</t>
+          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>HR Analyst</t>
+          <t>Forward Deployed Marketing Data Scientist</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote (North America)</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="G138" s="2" t="inlineStr">
-        <is>
-          <t>hr, analyst, system, training, technical, support</t>
-        </is>
-      </c>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr"/>
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>SurveyMonkey is the world's most popular platform for surveys and forms, built for businessâloved by users. We combine powerful capabilities with intuitive design, effectively serving every use case, from customer experience to employee engagement, market research to payment and registration forms. With built-in research expertise and AI-powered technology, it's like having a team of expert rese</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-hr-analyst-surveymonkey-1130353</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Forward Deployed Marketing Data Scientist</t>
+          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Remote (North America)</t>
+          <t>Remote-USA</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6395,26 +6399,26 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About Hightouch&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Hightouch is the modern AI platform for marketing and growth teams. Our AI agents reimagine marketing workflows, allowing marketers to create content, plan campaigns, and execute strategies with transformational velocity and performance.&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Hightouch is a rare compa</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5718912004</t>
+          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, Listings and Host Tools Data and AI</t>
+          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6429,7 +6433,7 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Remote-USA</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -6439,7 +6443,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr"/>
@@ -6451,14 +6455,14 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7454348?gh_jid=7454348</t>
+          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer - Community Support Engineering</t>
+          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6483,7 +6487,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="G141" t="inlineStr"/>
@@ -6495,19 +6499,19 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7116975?gh_jid=7116975</t>
+          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Senior Staff Machine Learning Engineer, Communication &amp; Connectivity</t>
+          <t>AI Applied Scientist</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -6517,7 +6521,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>San Francisco, CA • New York, NY • United States</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -6527,26 +6531,26 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-family: helvetica, arial, sans-serif; font-size: 12pt;&amp;quot;&amp;gt;Airbnb was born in 2007 when two hosts welcomed three guests to their San Francisco home, and has since grown to over 5 million hosts who have welcomed over 2 billion guest arrivals in almost every country across the globe. Every day, hosts offer unique stay</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>https://careers.airbnb.com/positions/7005605?gh_jid=7005605</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>AI Applied Scientist</t>
+          <t>People Analyst</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6583,14 +6587,14 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>People Analyst</t>
+          <t xml:space="preserve">Data Scientist  </t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -6615,7 +6619,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
@@ -6627,14 +6631,14 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5737300004?gh_jid=5737300004</t>
+          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Scientist  </t>
+          <t>Software Engineer, Machine Learning</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -6671,92 +6675,12 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/figma/jobs/5552580004?gh_jid=5552580004</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer, Machine Learning</t>
-        </is>
-      </c>
-      <c r="B146" s="2" t="inlineStr">
-        <is>
-          <t>Figma</t>
-        </is>
-      </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>San Francisco, CA • New York, NY • United States</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="G146" s="2" t="inlineStr"/>
-      <c r="H146" s="2" t="inlineStr"/>
-      <c r="I146" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;Figma is growing our team of passionate creatives and builders on a mission to make design accessible to all. Figma’s platform helps teams bring ideas to life—whether youre brainstorming, creating a prototype, translating designs into code, or iterating with AI. From idea to product, Figma empowers teams to streamline workflows, move faster, and </t>
-        </is>
-      </c>
-      <c r="J146" s="2" t="inlineStr">
-        <is>
           <t>https://boards.greenhouse.io/figma/jobs/5551532004?gh_jid=5551532004</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>Business Analyst (Loyalty/Retention)</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Mercuryo</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>❓ Unknown</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Himalayas</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>Hi! We're Mercuryo , and we're on a mission to redefine finance by blending the best of traditional banking with the power of decentralized finance (DeFi). We believe everyone deserves seamless access to Web3 and traditional financial services, so we're building the platform that makes it real: one that simplifies crypto and integrates it into the broader financial ecosystem. Since launching in 20</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J147"/>
+  <autoFilter ref="A1:J145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Auto-refresh: 2026-04-09 17:09 UTC
</commit_message>
<xml_diff>
--- a/job-monitor/job_monitor.xlsx
+++ b/job-monitor/job_monitor.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Listings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$J$144</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -826,27 +826,27 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Junior AI/ML Engineer (Data &amp; Cloud Platforms)</t>
+          <t>Senior Marketing Data Analyst</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mod Op</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -856,32 +856,36 @@
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-ai-ml-engineer-data-cloud-platforms-at-mod-op-4399859352</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7583474003</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Data Scientist, All Levels</t>
+          <t>Junior AI/ML Engineer (Data &amp; Cloud Platforms)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>Mod Op</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,24 +903,24 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4387600293</t>
+          <t>https://www.linkedin.com/jobs/view/junior-ai-ml-engineer-data-cloud-platforms-at-mod-op-4399859352</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist I</t>
+          <t>Data Scientist, All Levels</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Oscar Health</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -939,19 +943,19 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384795150</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-all-levels-at-ramp-4387600293</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ML Engineer</t>
+          <t>Data Scientist I</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Catalyst Labs</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -961,7 +965,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -979,19 +983,19 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ml-engineer-at-catalyst-labs-4398673366</t>
+          <t>https://www.linkedin.com/jobs/view/data-scientist-i-at-oscar-health-4384795150</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Junior Business Intelligence Analyst</t>
+          <t>ML Engineer</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Emerald Resource Group</t>
+          <t>Catalyst Labs</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1001,7 +1005,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Broadview Heights, OH</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1019,19 +1023,19 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/junior-business-intelligence-analyst-at-emerald-resource-group-4400208330</t>
+          <t>https://www.linkedin.com/jobs/view/ml-engineer-at-catalyst-labs-4398683222</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Data Analyst - Power BI Dashboard Development</t>
+          <t>Junior Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Accylerate</t>
+          <t>Emerald Resource Group</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1041,7 +1045,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Broadview Heights, OH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1059,58 +1063,54 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-power-bi-dashboard-development-at-accylerate-4399855505</t>
+          <t>https://www.linkedin.com/jobs/view/junior-business-intelligence-analyst-at-emerald-resource-group-4400208330</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Principal Sales Operations Analyst</t>
+          <t>Data Analyst - Power BI Dashboard Development</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Mongodb</t>
+          <t>Accylerate</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
-        </is>
-      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-power-bi-dashboard-development-at-accylerate-4399855505</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Senior Business Analyst, Technical Services</t>
+          <t>Principal Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1142,19 +1142,19 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
+          <t>&amp;lt;p&amp;gt;We’re looking for a driven individual with strong analytical instincts and a passion for turning data into actionable insights to support a rapidly growing Customer Success organization. In this role, you’ll guide the analytical rhythm of the business in partnership with CS leadership to surface trends, optimize segmentation and territories, and inform headcount and planning decisions. Yo</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7725834</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior Business Analyst, Technical Services</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1186,19 +1186,19 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
+          <t xml:space="preserve">&amp;lt;p&amp;gt;Partnering with stakeholders in the Technical Services (post-sales support) team, Analytics team, and other teams around the business, this role will surface key insights to drive business decision making. This role requires someone with strong analytical and technical skills, operational experience driving efficiencies, ability to apply a data-first mindset to strategic initiatives, and </t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=6841436</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Senior Data Analyst II, Growth</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1230,19 +1230,19 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
+          <t>&amp;lt;p&amp;gt;The worldwide data management software market is massive (According to IDC, the worldwide database software market, which it refers to as the database management systems software market, was forecasted to be approximately $82 billion in 2023 growing to approximately $137 billion in 2027. This represents a 14% compound annual growth rate). At MongoDB we are transforming industries and empo</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7696633</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Senior Sales Operations Analyst</t>
+          <t>Senior Data Analyst II, Growth</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Dublin</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1274,24 +1274,24 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
+          <t>&amp;lt;p&amp;gt;As a Senior Data Analyst II, Growth Analytics, you will be a critical contributor to MongoDB’s Product-Led-Growth business, becoming an expert in the middle and later stages of our relationship with customers to help identify and respond to changes in business performance and adjust our strategies accordingly. This is a highly visible role whose work will be directly leveraged at the exec</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7532424</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Marketing Insights Analyst</t>
+          <t>Senior Sales Operations Analyst</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fivetran</t>
+          <t>Mongodb</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Oakland, California, United States, AMER</t>
+          <t>Dublin</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1318,24 +1318,24 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
+          <t>&amp;lt;h3&amp;gt;The role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;To fuel this growth, we are hiring a Senior GTM Intelligence Analyst to build the data-driven analytics team. This role is a key member of our growing GTM Analytics team and is responsible for building and maintaining data infrastructure used by our global salesforce and leadership team, with a strong emphasis on stakeholder collaboration.&amp;lt;/p&amp;gt; &amp;lt;h3&amp;gt</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=7716912</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Staff Data Scientist, Product (Crypto)</t>
+          <t>Marketing Insights Analyst</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Fivetran</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY</t>
+          <t>Oakland, California, United States, AMER</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1362,24 +1362,24 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;From Fivetran’s founding until now, our mission has remained the same: to make access to data as simple and reliable as electricity. With Fivetran, customer data arrives in their warehouses, canonical and ready to query, with no engineering or maintenance required. We’re proud that more organizations continue to leverage our technology every day </t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
+          <t>https://www.fivetran.com/careers/job?gh_jid=7674622003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Data Analyst II</t>
+          <t>Staff Data Scientist, Product (Crypto)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Menlo Park, CA; New York, NY</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1406,19 +1406,19 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463696002?gh_jid=8463696002</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7489743?t=gh_src=&amp;gh_jid=7489743</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst III</t>
+          <t>Data Analyst II</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1455,14 +1455,14 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
+          <t>https://www.brex.com/careers/8463702002?gh_jid=8463702002</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Data Scientist, Finance </t>
+          <t>Data Analyst III</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, New York, United States</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1499,19 +1499,19 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
+          <t>https://www.brex.com/careers/8463704002?gh_jid=8463704002</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst, Financial Crimes &amp; Identity</t>
+          <t xml:space="preserve">Senior Data Scientist, Finance </t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Chime</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1538,19 +1538,19 @@
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
+          <t>https://www.brex.com/careers/7892186002?gh_jid=7892186002</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lead Data Analyst</t>
+          <t>Data Analyst, Financial Crimes &amp; Identity</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Chicago, IL, USA; San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1582,19 +1582,19 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h3&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;We are hiring for a Senior Analyst to drive data-informed risk strategy on our Financial Crimes &amp;amp; Identity team. As our Sr. Analyst, you will lead efforts to strengthen identity verification, customer onboarding, and lifecycle risk management by leveraging data to inform decisioning and control performance. You’ll partne</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8485895002?gh_jid=8485895002</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Lead Data Analyst, Growth Science</t>
+          <t>Lead Data Analyst</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1626,19 +1626,19 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403069002?gh_jid=8403069002</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Staff Data Analyst</t>
+          <t>Lead Data Analyst, Growth Science</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA; San Francisco, CA, USA; Seattle, WA, USA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1670,39 +1670,39 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+          <t>&amp;lt;h2&amp;gt;&amp;lt;strong&amp;gt;About the role&amp;lt;/strong&amp;gt;&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;We’re hiring a Lead Data Analyst, Growth Science to use advanced science to estimate the incrementality of Marketing, Product, and Lifecycle Marketing and to improve their performance. As a senior individual contributor, you’ll lead high-impact growth initiatives through the use of media mix modeling, experimentation and qua</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8462910002?gh_jid=8462910002</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Staff Data Analyst</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>SS&amp;C Technologies</t>
+          <t>Chime</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1712,22 +1712,26 @@
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;h3&amp;gt;About the Role&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;Chime is the largest and fastest-growing U.S. player in the challenger-banking space. Through our banking partners, we offer access to bank accounts with fee-free overdraft, provide members the chance to receive early access to their paychecks, help them improve their credit, and more. We created Chime because we believe everyone deserves financial peac</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
+          <t>https://boards.greenhouse.io/chime/jobs/8403065002?gh_jid=8403065002</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Data Analyst - Junior</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Global Technical Talent, an Inc. 5000 Company</t>
+          <t>SS&amp;C Technologies</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1737,7 +1741,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Framingham, MA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1755,19 +1759,19 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ss-c-technologies-4385100313</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Data Analyst - Junior</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>SeatGeek</t>
+          <t>Global Technical Talent, an Inc. 5000 Company</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1777,7 +1781,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Framingham, MA</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1795,7 +1799,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-junior-at-global-technical-talent-an-inc-5000-company-4398417362</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1811,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Betterment</t>
+          <t>SeatGeek</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1835,19 +1839,19 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-seatgeek-4384780557</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Engineer</t>
+          <t>Analytics Engineer</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Brain Co.</t>
+          <t>Betterment</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1857,7 +1861,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>San Francisco Bay Area</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1875,7 +1879,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-brain-co-4275844846</t>
+          <t>https://www.linkedin.com/jobs/view/analytics-engineer-at-betterment-4304721728</t>
         </is>
       </c>
     </row>
@@ -2082,51 +2086,47 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Senior Revenue Operations Analyst</t>
+          <t>Business Analyst, Life Sciences Strategy (NYC) Global Career Launchpad</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Brex</t>
+          <t>LSC - LifeSciences Consultants</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
-        </is>
-      </c>
+      <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8485385002?gh_jid=8485385002</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-life-sciences-strategy-nyc-global-career-launchpad-at-lsc-lifesciences-consultants-4399271713</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Product Data Platform</t>
+          <t>Senior Revenue Operations Analyst</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>San Francisco, California, United States</t>
+          <t>Seattle, Washington, United States</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2163,34 +2163,34 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
+          <t>https://www.brex.com/careers/8485386002?gh_jid=8485386002</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Senior Software Engineer, Product Data Platform</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>IMA Financial Group, Inc.</t>
+          <t>Brex</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>❓ Unknown</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Francisco, California, United States</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2200,22 +2200,26 @@
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;p&amp;gt;&amp;lt;strong&amp;gt;Why join us&amp;lt;/strong&amp;gt;&amp;lt;/p&amp;gt; &amp;lt;p&amp;gt;Brex is the intelligent finance platform that enables companies to spend smarter and move faster in more than 200 markets. By combining global corporate cards and banking with intuitive spend management, bill pay, and travel software, Brex enables founders and finance teams to accelerate</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
+          <t>https://www.brex.com/careers/8430182002?gh_jid=8430182002</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Entry Level Data Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>IMA Financial Group, Inc.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2225,7 +2229,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2243,19 +2247,19 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-ima-financial-group-inc-4398267799</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Entry Level Data Analyst</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Webologix Ltd/ INC</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2265,7 +2269,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2283,7 +2287,7 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-data-analyst-at-emonics-llc-4395458243</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2299,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>HirePower Staffing Solution</t>
+          <t>Webologix Ltd/ INC</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2305,7 +2309,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Fullerton, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2323,19 +2327,19 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-webologix-ltd-inc-4398543541</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Entry Level Machine Learning Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Emonics LLC</t>
+          <t>HirePower Staffing Solution</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2345,7 +2349,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Fullerton, CA</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2363,19 +2367,19 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-hirepower-staffing-solution-4398262716</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Business Intelligence (BI) Analyst</t>
+          <t>Entry Level Machine Learning Engineer</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GCON LLC</t>
+          <t>Emonics LLC</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2385,7 +2389,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2403,19 +2407,19 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
+          <t>https://www.linkedin.com/jobs/view/entry-level-machine-learning-engineer-at-emonics-llc-4395445490</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>CCAR Business Analyst</t>
+          <t>Business Intelligence (BI) Analyst</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Mitchell Martin Inc.</t>
+          <t>GCON LLC</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2425,7 +2429,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Jersey City, NJ</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2443,19 +2447,19 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
+          <t>https://www.linkedin.com/jobs/view/business-intelligence-bi-analyst-at-gcon-llc-4385609336</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>CCAR Business Analyst</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>The Allan Sullivan Co.</t>
+          <t>Mitchell Martin Inc.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2465,7 +2469,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Greater Chicago Area</t>
+          <t>Jersey City, NJ</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2483,19 +2487,19 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
+          <t>https://www.linkedin.com/jobs/view/ccar-business-analyst-at-mitchell-martin-inc-4398400044</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst II</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>WHOOP</t>
+          <t>The Allan Sullivan Co.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2505,7 +2509,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Greater Chicago Area</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2523,19 +2527,19 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-the-allan-sullivan-co-4398557857</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Analyst II</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Aditi Consulting</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2545,7 +2549,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Chillicothe, IL</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2563,19 +2567,19 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-ii-at-whoop-4398274131</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst, Digital Media</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Taboola</t>
+          <t>Aditi Consulting</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2585,7 +2589,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chillicothe, IL</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2603,7 +2607,7 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/business-analyst-digital-media-at-taboola-4398368627</t>
+          <t>https://www.linkedin.com/jobs/view/business-analyst-at-aditi-consulting-4398570725</t>
         </is>
       </c>
     </row>
@@ -2990,12 +2994,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning Infrastructure</t>
+          <t>Credit Business Analyst, Banking Fraud</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3005,7 +3009,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Seattle, San Francisco</t>
+          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3022,19 +3026,19 @@
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;h2&amp;gt;Who we are&amp;lt;/h2&amp;gt; &amp;lt;h3&amp;gt;About Stripe&amp;lt;/h3&amp;gt; &amp;lt;p&amp;gt;&amp;lt;span style=&amp;quot;font-weight: 400;&amp;quot;&amp;gt;Stripe is a financial infrastructure platform for businesses. Millions of companies—from the world’s largest enterprises to the most ambitious startups—use Stripe to accept payments, grow their revenue, and accelerate new business opportunities. Our mission is to increase the </t>
+          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=7746033</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Credit Business Analyst, Banking Fraud</t>
+          <t>Senior Data Scientist, ML (Incentives)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3049,7 +3053,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Menlo Park, CA; New York, NY; Washington, DC</t>
+          <t>Menlo Park, CA</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3071,14 +3075,14 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7513613?t=gh_src=&amp;gh_jid=7513613</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, ML (Incentives)</t>
+          <t>Senior Machine Learning Engineer, Agentic</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3093,7 +3097,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Menlo Park, CA</t>
+          <t>Bellevue, WA; Menlo Park, CA</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3115,34 +3119,34 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7596426?t=gh_src=&amp;gh_jid=7596426</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, Agentic</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>Prestige Staffing</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>✅ Yes</t>
+          <t>❓ Unknown</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Bellevue, WA; Menlo Park, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3152,26 +3156,22 @@
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&amp;lt;div class=&amp;quot;content-intro&amp;quot;&amp;gt;&amp;lt;h2&amp;gt;Join us in building the future of finance.&amp;lt;/h2&amp;gt; &amp;lt;p&amp;gt;Our mission is to democratize finance for all. &amp;lt;a href=&amp;quot;https://www.cerulli.com/press-releases/cerulli-anticipates-124-trillion-in-wealth-will-transfer-through-2048&amp;quot; target=&amp;quot;_blank&amp;quot;&amp;gt;An estimated $124 trillion of assets&amp;lt;/a&amp;gt; will be inherited by younger </t>
-        </is>
-      </c>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/robinhood/jobs/7121213?t=gh_src=&amp;gh_jid=7121213</t>
+          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Data &amp; Business Intelligence Analyst</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>Cypress HCM</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3199,19 +3199,19 @@
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/data-analyst-at-prestige-staffing-4372619451</t>
+          <t>https://www.linkedin.com/jobs/view/data-business-intelligence-analyst-at-cypress-hcm-4395795